<commit_message>
feat: keep every skill effect in the box using exact steps or step
keep every skill effect in the box using exact steps or step bounds
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_skill_text.xlsx
+++ b/mod_project/data_tables/qol_skill_text.xlsx
@@ -445,8 +445,8 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="76" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="84" customWidth="1" min="15" max="15"/>
     <col width="86" customWidth="1" min="16" max="16"/>
   </cols>
@@ -514,7 +514,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>First_To_Last_Only</t>
+          <t>Not_Level_By_Level</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -764,7 +764,7 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>ATK: 125% -&gt; 134 -&gt; 143 -&gt; 152 -&gt; 161 -&gt; 170 -&gt; 178 -&gt; 186 -&gt; 193 -&gt; 200% (L10)
-TP Cost: 5 -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 | Speed: 0.8x -&gt; 0.9x</t>
+Accuracy: +20% (+2%/Lv) | TP Cost: 5 (+2-3/Lv) -&gt; 28 | Speed: 0.8x -&gt; 0.9x</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -775,12 +775,12 @@
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
           <t>Short-range strike. | Hit Rate: +20% -&gt; +38% (+2%/Lv)</t>
@@ -831,7 +831,7 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>Accuracy: +20% -&gt; +22 -&gt; +24 -&gt; +26 -&gt; +28 -&gt; +30 -&gt; +31 -&gt; +32 -&gt; +33 -&gt; +35% (L10)
-TP Cost: 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 | Speed: 0.9x</t>
+Buff cancel rate: 68% (+1-2%/Lv) -&gt; 85% | TP Cost: 5 (+1-2/Lv) -&gt; 18 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -842,12 +842,12 @@
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Buff cancel rate</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Buff cancel rate, TP Cost</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
           <t>Short-range strike to one enemy. May cancel enemy active buffs.</t>
@@ -897,8 +897,8 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ATK: +20% -&gt; +30% -&gt; +40% -&gt; +45% -&gt; +50% (L1-5 Max) | DEF: -11% -&gt; -25%
-Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+          <t>ATK: +20% -&gt; +30% -&gt; +40% -&gt; +45% -&gt; +50% (L1-5 Max)
+DEF: -11% -&gt; -14% -&gt; -17% -&gt; -21% -&gt; -25% | Turns: 4 -&gt; 8 | TP Cost: 8 (+2/Lv) -&gt; 16</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -911,7 +911,7 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>Turns</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -968,8 +968,8 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>DEF: +20% -&gt; +30% -&gt; +40% -&gt; +45% -&gt; +50% (L1-5 Max) | ATK: -11% -&gt; -25%
-Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+          <t>DEF: +20% -&gt; +30% -&gt; +40% -&gt; +45% -&gt; +50% (L1-5 Max)
+ATK: -11% -&gt; -14% -&gt; -17% -&gt; -21% -&gt; -25% | Turns: 4 -&gt; 8 | TP Cost: 8 (+2/Lv) -&gt; 16</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -982,7 +982,7 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>Turns</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ATK: 85% -&gt; 90% -&gt; 94% -&gt; 98% -&gt; 102% (L1-5 Max) | Accuracy: +6% -&gt; +20%
+          <t>ATK: 85% -&gt; 90% -&gt; 94% -&gt; 98% -&gt; 102% (L1-5 Max) | Accuracy: +6% (+3-4%/Lv) -&gt; +20%
 Stun: 30% -&gt; 32% -&gt; 34% -&gt; 36% -&gt; 38% | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
@@ -1111,7 +1111,7 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>ATK: 106% -&gt; 112 -&gt; 118 -&gt; 124 -&gt; 130 -&gt; 134 -&gt; 138 -&gt; 142 -&gt; 146 -&gt; 150% (L10)
-TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 | Speed: 0.85x</t>
+Accuracy: +5% (+2-3%/Lv) -&gt; +28% | Paralysis: 20% -&gt; 50% | TP Cost: 6 (+2/Lv) -&gt; 24</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1122,10 +1122,14 @@
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Accuracy, Paralysis</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Accuracy, Paralysis</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1253,7 +1257,7 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>ATK: 80% -&gt; 83 -&gt; 86 -&gt; 89 -&gt; 91 -&gt; 94 -&gt; 97 -&gt; 100 -&gt; 105 -&gt; 110% (L10)
-TP Cost: 38 -&gt; 42 -&gt; 46 -&gt; 50 -&gt; 54 -&gt; 58 -&gt; 62 -&gt; 66 -&gt; 70 -&gt; 74</t>
+Instakill: 10% (+1-2%/Lv) -&gt; 20% | TP Cost: 38 (+4/Lv) -&gt; 74 | Speed: 0.65x -&gt; 0.75x</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1264,12 +1268,12 @@
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Instakill, Speed</t>
-        </is>
-      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Instakill</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
           <t>Katana skill. Deal slash damage to an enemy row. May instakill.</t>
@@ -1320,7 +1324,7 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>ATK: 84% -&gt; 88 -&gt; 92 -&gt; 96 -&gt; 100 -&gt; 104 -&gt; 108 -&gt; 112 -&gt; 116 -&gt; 120% (L10)
-Turns: 4 | TP Cost: 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30 -&gt; 32</t>
+Enemy DEF: -16% (-1%/Lv) | Turns: 4 | TP Cost: 14 (+2/Lv) -&gt; 32 | Speed: 0.8x</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1332,11 +1336,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Enemy DEF, Speed</t>
-        </is>
-      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
           <t>Katana skill. Deal defense-piercing damage and lower target DEF.</t>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ATK: 74% -&gt; 78 -&gt; 82 -&gt; 86 -&gt; 90 -&gt; 94 -&gt; 98 -&gt; 102 -&gt; 106 -&gt; 110% (L10)
+          <t>ATK: 74% (+4%/Lv) -&gt; 110% (L10 Max) | HP Absorb: 15% (+1-2%/Lv) -&gt; 25%
 TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 36 | Speed: 0.9x</t>
         </is>
       </c>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>HP Absorb</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>Short-range strike to one enemy. Absorb a portion of damage as HP.</t>
@@ -1588,7 +1588,7 @@
       <c r="H17" t="inlineStr">
         <is>
           <t>ATK: 65% -&gt; 70 -&gt; 75 -&gt; 80 -&gt; 84 -&gt; 88 -&gt; 91 -&gt; 94 -&gt; 97 -&gt; 100% (L10)
-TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 | Speed: 0.9x</t>
+TP Absorb: 10% (+1-2%/Lv) -&gt; 20% | TP Cost: 6 (+2/Lv) -&gt; 24 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1599,12 +1599,12 @@
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>TP Absorb</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>Short-range strike to one enemy. Absorb a portion of damage as TP.</t>
@@ -1655,7 +1655,7 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>ATK: 130% -&gt; 144 -&gt; 157 -&gt; 170 -&gt; 182 -&gt; 194 -&gt; 204 -&gt; 212 -&gt; 220 -&gt; 228% (L10)
-Freeze: 20% -&gt; 50% | TP Cost: 9 -&gt; 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36</t>
+Freeze: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 9 (+3/Lv) -&gt; 36 | Speed: 0.75x -&gt; 0.85x</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1671,11 +1671,7 @@
           <t>Freeze</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
           <t>Short-range strike dealing mid-range water damage. May freeze.</t>
@@ -1726,7 +1722,7 @@
       <c r="H19" t="inlineStr">
         <is>
           <t>ATK: 135% -&gt; 149 -&gt; 163 -&gt; 176 -&gt; 189 -&gt; 201 -&gt; 213 -&gt; 225 -&gt; 236 -&gt; 247% (L10)
-TP Cost: 9 -&gt; 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 37 -&gt; 42</t>
+Petrify: 20% (+1-2%/Lv) -&gt; 35% | TP Cost: 9 (+3-5/Lv) -&gt; 42 | Speed: 0.85x -&gt; 0.95x</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1737,12 +1733,12 @@
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Petrify, Speed</t>
-        </is>
-      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Petrify, TP Cost</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>Axe skill. Strike one enemy with earth damage. May petrify.</t>
@@ -1793,7 +1789,7 @@
       <c r="H20" t="inlineStr">
         <is>
           <t>ATK: 120% -&gt; 130 -&gt; 140 -&gt; 148 -&gt; 156 -&gt; 164 -&gt; 170 -&gt; 176 -&gt; 180 -&gt; 184% (L10)
-Targets: 2 -&gt; 5 | TP Cost: 26 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 47 -&gt; 53 -&gt; 58 -&gt; 63 -&gt; 68</t>
+Targets: 2 -&gt; 2 -&gt; 2 -&gt; 3 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 5 -&gt; 5 | TP Cost: 26 (+4-6/Lv) -&gt; 68</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1806,7 +1802,7 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Targets</t>
+          <t>TP Cost</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1998,7 +1994,7 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>ATK: 130% -&gt; 140 -&gt; 150 -&gt; 160 -&gt; 170 -&gt; 180 -&gt; 190 -&gt; 200 -&gt; 211 -&gt; 222% (L10)
-TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 39</t>
+Accuracy: +6% (+1-2%/Lv) -&gt; +20% | TP Cost: 12 (+3/Lv) -&gt; 39 | Speed: 0.8x -&gt; 0.9x</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -2009,12 +2005,12 @@
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Accuracy, Speed</t>
-        </is>
-      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>Sword and lance skill. Strike one enemy. Effective vs. Unholy foes.</t>
@@ -2199,7 +2195,7 @@
       <c r="H26" t="inlineStr">
         <is>
           <t>ATK: 96% -&gt; 100 -&gt; 104 -&gt; 108 -&gt; 113 -&gt; 118 -&gt; 123 -&gt; 128 -&gt; 133 -&gt; 138% (L10)
-TP Cost: 26 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 -&gt; 54 -&gt; 59 -&gt; 64 | Speed: 0.8x</t>
+Paralysis: 20% (+2-3%/Lv) -&gt; 40% | TP Cost: 26 (+4-5/Lv) -&gt; 64 | Speed: 0.8x</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -2210,12 +2206,12 @@
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Paralysis</t>
-        </is>
-      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Paralysis, TP Cost</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>Short-range skill. Deal lightning damage to an enemy row. May paralyze.</t>
@@ -2266,7 +2262,7 @@
       <c r="H27" t="inlineStr">
         <is>
           <t>ATK: 135% -&gt; 149 -&gt; 163 -&gt; 176 -&gt; 189 -&gt; 201 -&gt; 213 -&gt; 223 -&gt; 234 -&gt; 245% (L10)
-TP Cost: 7 -&gt; 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22 -&gt; 25 -&gt; 28 -&gt; 31 -&gt; 34</t>
+Silence: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 7 (+3/Lv) -&gt; 34 | Speed: 0.85x -&gt; 0.95x</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -2277,12 +2273,12 @@
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Silence, Speed</t>
-        </is>
-      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Silence</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>Lance skill. Strike one enemy with wind damage. May silence.</t>
@@ -2400,7 +2396,7 @@
       <c r="H29" t="inlineStr">
         <is>
           <t>ATK: 120% -&gt; 130 -&gt; 142 -&gt; 154 -&gt; 165 -&gt; 176 -&gt; 186 -&gt; 196 -&gt; 204 -&gt; 212% (L10)
-TP Cost: 32 -&gt; 35 -&gt; 38 -&gt; 41 -&gt; 44 -&gt; 47 -&gt; 50 -&gt; 53 -&gt; 56 -&gt; 59 | Speed: 0.8x</t>
+Accuracy: +5% (+1-2%/Lv) -&gt; +15% | TP Cost: 32 (+3/Lv) -&gt; 59 | Speed: 0.8x</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -2411,12 +2407,12 @@
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>Accuracy</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
           <t>Sword and lance skill. Pierces through to the back row.</t>
@@ -2993,7 +2989,7 @@
       <c r="H38" t="inlineStr">
         <is>
           <t>Speed increase: 10% -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15 -&gt; 16 -&gt; 17 -&gt; 18 -&gt; 20% (L10)
-Turns: 3 -&gt; 6 | TP Cost: 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30 -&gt; 32</t>
+Turns: 3 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 5 -&gt; 5 -&gt; 5 -&gt; 6 | TP Cost: 14 (+2/Lv) -&gt; 32</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -3004,11 +3000,7 @@
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>Turns</t>
-        </is>
-      </c>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
@@ -3135,7 +3127,7 @@
       <c r="H40" t="inlineStr">
         <is>
           <t>ATK: 116% -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 150 -&gt; 156% (L10)
-TP Cost: 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25 | Speed: 0.9x</t>
+Sleep: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 7 (+2/Lv) -&gt; 25 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -3146,12 +3138,12 @@
       </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>Sleep</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
           <t>Short-range strike to one enemy. May inflict Sleep.</t>
@@ -3202,7 +3194,7 @@
       <c r="H41" t="inlineStr">
         <is>
           <t>ATK: 116% -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 150 -&gt; 156% (L10)
-TP Cost: 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25 | Speed: 0.9x</t>
+Silence: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 7 (+2/Lv) -&gt; 25 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -3213,12 +3205,12 @@
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>Silence</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
           <t>Short-range strike to one enemy. May inflict Silence.</t>
@@ -3269,7 +3261,7 @@
       <c r="H42" t="inlineStr">
         <is>
           <t>ATK: 112% -&gt; 116 -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 150% (L10)
-TP Cost: 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25 | Speed: 0.9x</t>
+Stun: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 7 (+2/Lv) -&gt; 25 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -3280,12 +3272,12 @@
       </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>Stun</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
           <t>Short-range strike to one enemy. May inflict Stun.</t>
@@ -3336,7 +3328,7 @@
       <c r="H43" t="inlineStr">
         <is>
           <t>Number of attacks: 3 -&gt; 3 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 5 -&gt; 5 | ATK: 104% -&gt; 148%
-TP Cost: 30 -&gt; 34 -&gt; 38 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 58 -&gt; 64 -&gt; 68 -&gt; 72</t>
+Power: -25% -&gt; -14% | TP Cost: 30 (+4-6/Lv) -&gt; 72 | Speed: 0.75x -&gt; 0.85x</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -3349,14 +3341,10 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
-          <t>ATK</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Power, Speed</t>
-        </is>
-      </c>
+          <t>ATK, Power, TP Cost</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
           <t>Bow and gun skill. Rapid fire multiple shots with escalating crit rate.</t>
@@ -3541,7 +3529,7 @@
       <c r="H46" t="inlineStr">
         <is>
           <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170% (L10)
-Poison: 20% -&gt; 50% | TP Cost: 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25</t>
+Poison: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 7 (+2/Lv) -&gt; 25</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -3608,7 +3596,7 @@
       <c r="H47" t="inlineStr">
         <is>
           <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170% (L10)
-Freeze: 20% -&gt; 50% | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26</t>
+Freeze: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 8 (+2/Lv) -&gt; 26</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -3675,7 +3663,7 @@
       <c r="H48" t="inlineStr">
         <is>
           <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170% (L10)
-TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26</t>
+Paralysis: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 8 (+2/Lv) -&gt; 26</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -3686,12 +3674,12 @@
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>Paralysis</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr">
         <is>
           <t>Bow skill. Attack one enemy with an electric shot. May paralyze.</t>
@@ -3742,7 +3730,7 @@
       <c r="H49" t="inlineStr">
         <is>
           <t>ATK: 116% -&gt; 122 -&gt; 128 -&gt; 134 -&gt; 140 -&gt; 145 -&gt; 150 -&gt; 155 -&gt; 160 -&gt; 165% (L10)
-TP Cost: 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25 -&gt; 27 | Speed: 0.95x</t>
+Slow: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 9 (+2/Lv) -&gt; 27 | Speed: 0.95x</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -3753,12 +3741,12 @@
       </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>Slow</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
           <t>Bow skill. Deal stab damage to one enemy. May slow.</t>
@@ -3943,7 +3931,7 @@
       <c r="H52" t="inlineStr">
         <is>
           <t>ATK: 130% -&gt; 144 -&gt; 158 -&gt; 171 -&gt; 184 -&gt; 196 -&gt; 207 -&gt; 217 -&gt; 226 -&gt; 234% (L10)
-TP Cost: 24 -&gt; 28 -&gt; 32 -&gt; 36 -&gt; 40 -&gt; 43 -&gt; 46 -&gt; 49 -&gt; 52 -&gt; 55 | Speed: 0.7x</t>
+Critical rate: 5 (+1-3/Lv) -&gt; 25 | TP Cost: 24 (+3-4/Lv) -&gt; 55 | Speed: 0.7x</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -3954,12 +3942,12 @@
       </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>Critical rate</t>
-        </is>
-      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Critical rate, TP Cost</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr">
         <is>
           <t>Bow skill. Massive piercing shot that penetrates through to the back row.</t>
@@ -4072,7 +4060,7 @@
       <c r="H54" t="inlineStr">
         <is>
           <t>ATK: 120% -&gt; 126 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 154 -&gt; 162 -&gt; 170 -&gt; 180 -&gt; 192% (L10)
-TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 36 | Speed: 0.45x</t>
+Stun: 10% -&gt; 20% | TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 36</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -4083,10 +4071,14 @@
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Stun</t>
+        </is>
+      </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Stun</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -4201,7 +4193,7 @@
       <c r="H56" t="inlineStr">
         <is>
           <t>Magic damage: +38% -&gt; +42% -&gt; +47% -&gt; +53% -&gt; +60% (L1-5 Max)
-Turns: 6 | TP Cost: 20 -&gt; 23 -&gt; 26 -&gt; 29 -&gt; 32 | Speed: 1.5x -&gt; 2.1x</t>
+Magic accuracy: -2% (-2%/Lv) | Turns: 6 | TP Cost: 20 -&gt; 23 -&gt; 26 -&gt; 29 -&gt; 32</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -4215,7 +4207,7 @@
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Magic accuracy</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
@@ -4258,7 +4250,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Accuracy: +10% -&gt; +12 -&gt; +14 -&gt; +16 -&gt; +18 -&gt; +20 -&gt; +22 -&gt; +24 -&gt; +26 -&gt; +30% (L10)
+          <t>Damage UP | Accuracy: +10% (+2-4%/Lv) -&gt; +30%
 TP Cost: 28 -&gt; 32 -&gt; 36 -&gt; 40 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 56 -&gt; 60 -&gt; 64 | Speed: 0.75x</t>
         </is>
       </c>
@@ -4278,12 +4270,12 @@
           <t>effect_3</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>Damage UP</t>
-        </is>
-      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr">
         <is>
           <t>Mace skill. Heavy bash strike with boosted accuracy.</t>
@@ -4593,7 +4585,7 @@
       <c r="H62" t="inlineStr">
         <is>
           <t>ATK: 136% -&gt; 142 -&gt; 148 -&gt; 155 -&gt; 162 -&gt; 172 -&gt; 182 -&gt; 193 -&gt; 204 -&gt; 216% (L10)
-TP Cost: 13 -&gt; 16 -&gt; 19 -&gt; 22 -&gt; 25 -&gt; 29 -&gt; 33 -&gt; 37 -&gt; 41 -&gt; 45 | Speed: 0.9x -&gt; 1x</t>
+Accuracy: +10% (+1-2%/Lv) -&gt; +20% | TP Cost: 13 (+3-4/Lv) -&gt; 45 | Speed: 0.9x -&gt; 1x</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -4604,12 +4596,12 @@
       </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr">
         <is>
           <t>Short-range strike dealing heavy lightning damage to one enemy.</t>
@@ -4660,7 +4652,7 @@
       <c r="H63" t="inlineStr">
         <is>
           <t>ATK: 150% -&gt; 162 -&gt; 174 -&gt; 186 -&gt; 198 -&gt; 208 -&gt; 218 -&gt; 228 -&gt; 236 -&gt; 244% (L10)
-Freeze: 20% -&gt; 50% | TP Cost: 9 -&gt; 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36</t>
+Freeze: 20% (+3-4%/Lv) -&gt; 50% | Silence: 20% -&gt; 50% | TP Cost: 9 (+3/Lv) -&gt; 36</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -4673,14 +4665,10 @@
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Freeze</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>Silence</t>
-        </is>
-      </c>
+          <t>Freeze, Silence</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
     </row>
@@ -5879,7 +5867,7 @@
       <c r="H84" t="inlineStr">
         <is>
           <t>ATK: 120% -&gt; 126 -&gt; 132 -&gt; 138 -&gt; 142 -&gt; 150 -&gt; 158 -&gt; 168 -&gt; 178 -&gt; 190% (L10)
-TP Cost: 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25 -&gt; 27 -&gt; 29 -&gt; 31 -&gt; 33 -&gt; 35 | Speed: 0.88x</t>
+Instakill: 15% (+1-2%/Lv) -&gt; 25% | TP Cost: 17 (+2/Lv) -&gt; 35 | Speed: 0.88x</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -5890,12 +5878,12 @@
       </c>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr">
+      <c r="M84" t="inlineStr">
         <is>
           <t>Instakill</t>
         </is>
       </c>
+      <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr">
         <is>
           <t>Attack one enemy. May instakill.</t>
@@ -5946,7 +5934,7 @@
       <c r="H85" t="inlineStr">
         <is>
           <t>ATK: 95% -&gt; 99 -&gt; 103 -&gt; 107 -&gt; 111 -&gt; 115 -&gt; 119 -&gt; 123 -&gt; 127 -&gt; 131% (L10)
-TP Cost: 32 -&gt; 34 -&gt; 36 -&gt; 38 -&gt; 40 -&gt; 42 -&gt; 44 -&gt; 46 -&gt; 48 -&gt; 50 | Speed: 0.65x</t>
+Stun: 40% (+3-4%/Lv) -&gt; 70% | TP Cost: 32 (+2/Lv) -&gt; 50 | Speed: 0.65x</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -5957,12 +5945,12 @@
       </c>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr">
+      <c r="M85" t="inlineStr">
         <is>
           <t>Stun</t>
         </is>
       </c>
+      <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
     </row>
@@ -6003,7 +5991,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>ATK: 15% -&gt; 20% -&gt; 25% -&gt; 30% -&gt; 35% (L1-5 Max) | DEF: -11% -&gt; -25%
+          <t>ATK: 15% (+5%/Lv) -&gt; 35% (L5 Max) | DEF: -11% -&gt; -14% -&gt; -17% -&gt; -21% -&gt; -25%
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
@@ -6015,11 +6003,7 @@
       </c>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>DEF</t>
-        </is>
-      </c>
+      <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr">
         <is>
           <t>Speed</t>
@@ -6173,7 +6157,7 @@
       <c r="H89" t="inlineStr">
         <is>
           <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 164 -&gt; 170 -&gt; 176% (L10)
-TP Cost: 22 -&gt; 26 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 -&gt; 54 -&gt; 58</t>
+Poison: 50% (+3-4%/Lv) -&gt; 80% | TP Cost: 22 (+4/Lv) -&gt; 58 | Speed: 0.6x -&gt; 0.7x</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -6184,12 +6168,12 @@
       </c>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr">
-        <is>
-          <t>Poison, Speed</t>
-        </is>
-      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Poison</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr"/>
     </row>
@@ -6231,7 +6215,7 @@
       <c r="H90" t="inlineStr">
         <is>
           <t>ATK: 150% -&gt; 162 -&gt; 174 -&gt; 186 -&gt; 198 -&gt; 208 -&gt; 218 -&gt; 228 -&gt; 240 -&gt; 256% (L10)
-TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 23 -&gt; 26 -&gt; 29 -&gt; 32 | Speed: 0.95x</t>
+Turn delay rate: 25% (+2%/Lv) | TP Cost: 10 (+2-3/Lv) -&gt; 32 | Speed: 0.95x</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -6242,12 +6226,12 @@
       </c>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr">
-        <is>
-          <t>Turn delay rate</t>
-        </is>
-      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr">
         <is>
           <t>Fan skill. Deal bash damage to one enemy and delay target turn.</t>
@@ -9308,7 +9292,7 @@
       <c r="H145" t="inlineStr">
         <is>
           <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
-TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 | Speed: 2.25x</t>
+Accuracy: 86% (+1%/Lv) | TP Cost: 5 (+2-4/Lv) -&gt; 32 | Speed: 2.25x</t>
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
@@ -9319,10 +9303,14 @@
       </c>
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
-      <c r="M145" t="inlineStr"/>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -9375,7 +9363,7 @@
       <c r="H146" t="inlineStr">
         <is>
           <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
-TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 | Speed: 1.7x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 15 (+4-6/Lv) -&gt; 60 | Speed: 1.7x</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -9386,10 +9374,14 @@
       </c>
       <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr"/>
-      <c r="M146" t="inlineStr"/>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -9442,7 +9434,7 @@
       <c r="H147" t="inlineStr">
         <is>
           <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
-TP Cost: 42 -&gt; 50 -&gt; 58 -&gt; 64 -&gt; 73 -&gt; 82 -&gt; 91 -&gt; 100 -&gt; 110 -&gt; 120 | Speed: 1.3x</t>
+Accuracy: 75% (+1-2%/Lv) -&gt; 85% | TP Cost: 42 (+6-10/Lv) -&gt; 120 | Speed: 1.3x</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -9453,10 +9445,14 @@
       </c>
       <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr"/>
-      <c r="M147" t="inlineStr"/>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -9572,7 +9568,7 @@
       <c r="H149" t="inlineStr">
         <is>
           <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
-TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 | Speed: 2.25x</t>
+Accuracy: 86% (+1%/Lv) | TP Cost: 5 (+2-4/Lv) -&gt; 32 | Speed: 2.25x</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -9583,10 +9579,14 @@
       </c>
       <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr"/>
-      <c r="M149" t="inlineStr"/>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -9639,7 +9639,7 @@
       <c r="H150" t="inlineStr">
         <is>
           <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
-TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 | Speed: 1.7x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 15 (+4-6/Lv) -&gt; 60 | Speed: 1.7x</t>
         </is>
       </c>
       <c r="I150" t="inlineStr"/>
@@ -9650,10 +9650,14 @@
       </c>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
-      <c r="M150" t="inlineStr"/>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -9706,7 +9710,7 @@
       <c r="H151" t="inlineStr">
         <is>
           <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
-TP Cost: 42 -&gt; 50 -&gt; 58 -&gt; 64 -&gt; 73 -&gt; 82 -&gt; 91 -&gt; 100 -&gt; 110 -&gt; 120 | Speed: 1.3x</t>
+Accuracy: 75% (+1-2%/Lv) -&gt; 85% | TP Cost: 42 (+6-10/Lv) -&gt; 120 | Speed: 1.3x</t>
         </is>
       </c>
       <c r="I151" t="inlineStr"/>
@@ -9717,10 +9721,14 @@
       </c>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr"/>
-      <c r="M151" t="inlineStr"/>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -9836,7 +9844,7 @@
       <c r="H153" t="inlineStr">
         <is>
           <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
-TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 | Speed: 2.25x</t>
+Accuracy: 86% (+1%/Lv) | TP Cost: 5 (+2-4/Lv) -&gt; 32 | Speed: 2.25x</t>
         </is>
       </c>
       <c r="I153" t="inlineStr"/>
@@ -9847,10 +9855,14 @@
       </c>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
-      <c r="M153" t="inlineStr"/>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -9903,7 +9915,7 @@
       <c r="H154" t="inlineStr">
         <is>
           <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
-TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 | Speed: 1.7x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 15 (+4-6/Lv) -&gt; 60 | Speed: 1.7x</t>
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
@@ -9914,10 +9926,14 @@
       </c>
       <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr"/>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -9970,7 +9986,7 @@
       <c r="H155" t="inlineStr">
         <is>
           <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
-TP Cost: 42 -&gt; 50 -&gt; 58 -&gt; 64 -&gt; 73 -&gt; 82 -&gt; 91 -&gt; 100 -&gt; 110 -&gt; 120 | Speed: 1.3x</t>
+Accuracy: 75% (+1-2%/Lv) -&gt; 85% | TP Cost: 42 (+6-10/Lv) -&gt; 120 | Speed: 1.3x</t>
         </is>
       </c>
       <c r="I155" t="inlineStr"/>
@@ -9981,10 +9997,14 @@
       </c>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
-      <c r="M155" t="inlineStr"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -10100,7 +10120,7 @@
       <c r="H157" t="inlineStr">
         <is>
           <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
-TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 | Speed: 2.25x</t>
+Accuracy: 86% (+1%/Lv) | TP Cost: 5 (+2-4/Lv) -&gt; 32 | Speed: 2.25x</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -10111,10 +10131,14 @@
       </c>
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr"/>
-      <c r="M157" t="inlineStr"/>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -10167,7 +10191,7 @@
       <c r="H158" t="inlineStr">
         <is>
           <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
-TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 | Speed: 1.7x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 15 (+4-6/Lv) -&gt; 60 | Speed: 1.7x</t>
         </is>
       </c>
       <c r="I158" t="inlineStr"/>
@@ -10178,10 +10202,14 @@
       </c>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr"/>
-      <c r="M158" t="inlineStr"/>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -10234,7 +10262,7 @@
       <c r="H159" t="inlineStr">
         <is>
           <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
-TP Cost: 42 -&gt; 50 -&gt; 58 -&gt; 64 -&gt; 73 -&gt; 82 -&gt; 91 -&gt; 100 -&gt; 110 -&gt; 120 | Speed: 1.3x</t>
+Accuracy: 75% (+1-2%/Lv) -&gt; 85% | TP Cost: 42 (+6-10/Lv) -&gt; 120 | Speed: 1.3x</t>
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
@@ -10245,10 +10273,14 @@
       </c>
       <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr"/>
-      <c r="M159" t="inlineStr"/>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -10364,7 +10396,7 @@
       <c r="H161" t="inlineStr">
         <is>
           <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
-TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 | Speed: 2.25x</t>
+Accuracy: 86% (+1%/Lv) | TP Cost: 5 (+2-4/Lv) -&gt; 32 | Speed: 2.25x</t>
         </is>
       </c>
       <c r="I161" t="inlineStr"/>
@@ -10375,10 +10407,14 @@
       </c>
       <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr"/>
-      <c r="M161" t="inlineStr"/>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -10431,7 +10467,7 @@
       <c r="H162" t="inlineStr">
         <is>
           <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
-TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 | Speed: 1.7x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 15 (+4-6/Lv) -&gt; 60 | Speed: 1.7x</t>
         </is>
       </c>
       <c r="I162" t="inlineStr"/>
@@ -10442,10 +10478,14 @@
       </c>
       <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr"/>
-      <c r="M162" t="inlineStr"/>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -10498,7 +10538,7 @@
       <c r="H163" t="inlineStr">
         <is>
           <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
-TP Cost: 42 -&gt; 50 -&gt; 58 -&gt; 64 -&gt; 73 -&gt; 82 -&gt; 91 -&gt; 100 -&gt; 110 -&gt; 120 | Speed: 1.3x</t>
+Accuracy: 75% (+1-2%/Lv) -&gt; 85% | TP Cost: 42 (+6-10/Lv) -&gt; 120 | Speed: 1.3x</t>
         </is>
       </c>
       <c r="I163" t="inlineStr"/>
@@ -10509,10 +10549,14 @@
       </c>
       <c r="K163" t="inlineStr"/>
       <c r="L163" t="inlineStr"/>
-      <c r="M163" t="inlineStr"/>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -10628,7 +10672,7 @@
       <c r="H165" t="inlineStr">
         <is>
           <t>Pwr: 60 -&gt; 95 -&gt; 130 -&gt; 165 -&gt; 200 -&gt; 230 -&gt; 260 -&gt; 290 -&gt; 320 -&gt; 350 (L10)
-TP Cost: 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15 -&gt; 16 -&gt; 17 -&gt; 18 | Speed: 2x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 9 (+1/Lv) -&gt; 18 | Speed: 2x</t>
         </is>
       </c>
       <c r="I165" t="inlineStr"/>
@@ -10639,10 +10683,14 @@
       </c>
       <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -10833,7 +10881,7 @@
       <c r="H168" t="inlineStr">
         <is>
           <t>Pwr: 75 -&gt; 120 -&gt; 165 -&gt; 210 -&gt; 255 -&gt; 295 -&gt; 335 -&gt; 375 -&gt; 415 -&gt; 450 (L10)
-TP Cost: 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 | Speed: 1.5x</t>
+Accuracy: 65% (+2-3%/Lv) -&gt; 87% | TP Cost: 18 (+3-4/Lv) -&gt; 50 | Speed: 1.5x</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -10844,10 +10892,14 @@
       </c>
       <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -11584,7 +11636,7 @@
       <c r="H180" t="inlineStr">
         <is>
           <t>Pwr: 250 -&gt; 300 -&gt; 350 -&gt; 400 -&gt; 440 -&gt; 480 -&gt; 520 -&gt; 560 -&gt; 600 -&gt; 640 (L10)
-TP Cost: 45 -&gt; 52 -&gt; 59 -&gt; 66 -&gt; 74 -&gt; 80 -&gt; 86 -&gt; 90 -&gt; 95 -&gt; 100 | Speed: 1.75x</t>
+Accuracy: 60% (+1-2%/Lv) -&gt; 70% | TP Cost: 45 (+4-8/Lv) -&gt; 100 | Speed: 1.75x</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -11595,10 +11647,14 @@
       </c>
       <c r="K180" t="inlineStr"/>
       <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Accuracy, TP Cost</t>
+        </is>
+      </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O180" t="inlineStr"/>
@@ -12157,7 +12213,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>HP recovery: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 (L10)
+          <t>HP recovery: 8 (+2/Lv) -&gt; 26 (L10 Max) | Heal Cap: 100 (+60-80/Lv) -&gt; 800
 TP Cost: 3 -&gt; 5 -&gt; 7 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 | Speed: 1.75x</t>
         </is>
       </c>
@@ -12169,10 +12225,14 @@
       </c>
       <c r="K189" t="inlineStr"/>
       <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr"/>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Heal Cap</t>
+        </is>
+      </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>Heal Cap, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -12224,7 +12284,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>HP recovery: 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 (L10)
+          <t>HP recovery: 5 (+1/Lv) -&gt; 14 (L10 Max) | Heal Cap: 80 (+50-60/Lv) -&gt; 600
 TP Cost: 15 -&gt; 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 -&gt; 46 -&gt; 52 -&gt; 58 -&gt; 64 | Speed: 1.35x</t>
         </is>
       </c>
@@ -12236,10 +12296,14 @@
       </c>
       <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr"/>
-      <c r="M190" t="inlineStr"/>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Heal Cap</t>
+        </is>
+      </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>Heal Cap, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -12885,7 +12949,7 @@
       <c r="H200" t="inlineStr">
         <is>
           <t>Max HP: +20% -&gt; +23 -&gt; +26 -&gt; +29 -&gt; +32 -&gt; +35 -&gt; +38 -&gt; +41 -&gt; +44 -&gt; +47% (L10)
-Turns: 5 -&gt; 10 | TP Cost: 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 39 -&gt; 42 -&gt; 45</t>
+Turns: 5 -&gt; 5 -&gt; 6 -&gt; 6 -&gt; 7 -&gt; 7 -&gt; 8 -&gt; 8 -&gt; 9 -&gt; 10 | TP Cost: 18 (+3/Lv) -&gt; 45</t>
         </is>
       </c>
       <c r="I200" t="inlineStr"/>
@@ -12896,11 +12960,7 @@
       </c>
       <c r="K200" t="inlineStr"/>
       <c r="L200" t="inlineStr"/>
-      <c r="M200" t="inlineStr">
-        <is>
-          <t>Turns</t>
-        </is>
-      </c>
+      <c r="M200" t="inlineStr"/>
       <c r="N200" t="inlineStr">
         <is>
           <t>Speed, Chant</t>
@@ -14117,8 +14177,8 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | Damage cap UP
-Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x | Chant: 1x -&gt; 1.25x</t>
+          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | ATK: -4% (-1%/Lv)
+Damage cap UP | Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I221" t="inlineStr"/>
@@ -14140,7 +14200,7 @@
       <c r="M221" t="inlineStr"/>
       <c r="N221" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O221" t="inlineStr"/>
@@ -14183,8 +14243,8 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | Damage cap UP
-Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x | Chant: 1x -&gt; 1.25x</t>
+          <t>Damage UP | Accuracy: 64% (+4%/Lv) -&gt; 80% (L5 Max) | Magic defense: -7% -&gt; -18%
+Damage cap UP | Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I222" t="inlineStr"/>
@@ -14203,10 +14263,14 @@
           <t>effect_1, effect_3</t>
         </is>
       </c>
-      <c r="M222" t="inlineStr"/>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Magic defense</t>
+        </is>
+      </c>
       <c r="N222" t="inlineStr">
         <is>
-          <t>Magic defense</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O222" t="inlineStr"/>
@@ -14249,8 +14313,8 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | Damage cap UP
-Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x | Chant: 1x -&gt; 1.25x</t>
+          <t>Damage UP | Accuracy: 64% (+4%/Lv) -&gt; 80% (L5 Max) | Speed decrease: 4% (+1%/Lv)
+Damage cap UP | Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I223" t="inlineStr"/>
@@ -14272,7 +14336,7 @@
       <c r="M223" t="inlineStr"/>
       <c r="N223" t="inlineStr">
         <is>
-          <t>Speed decrease</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O223" t="inlineStr"/>
@@ -14315,8 +14379,8 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | Damage cap UP
-Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x | Chant: 1x -&gt; 1.25x</t>
+          <t>Damage UP | Accuracy: 64% (+4%/Lv) -&gt; 80% (L5 Max) | Evasion: -7% (-2%/Lv)
+Damage cap UP | Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
@@ -14338,7 +14402,7 @@
       <c r="M224" t="inlineStr"/>
       <c r="N224" t="inlineStr">
         <is>
-          <t>Evasion</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O224" t="inlineStr"/>
@@ -14381,8 +14445,8 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | Damage cap UP
-Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x | Chant: 1x -&gt; 1.25x</t>
+          <t>Damage UP | Accuracy: 64% -&gt; 68% -&gt; 72% -&gt; 76% -&gt; 80% (L1-5 Max) | DEF: -4% (-1%/Lv)
+Damage cap UP | Turns: 3 | TP Cost: 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I225" t="inlineStr"/>
@@ -14404,7 +14468,7 @@
       <c r="M225" t="inlineStr"/>
       <c r="N225" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O225" t="inlineStr"/>
@@ -14448,7 +14512,7 @@
       <c r="H226" t="inlineStr">
         <is>
           <t>Pwr: 350 -&gt; 390 -&gt; 430 -&gt; 470 -&gt; 510 -&gt; 550 -&gt; 590 -&gt; 630 -&gt; 680 -&gt; 720 (L10)
-TP Cost: 22 -&gt; 28 -&gt; 34 -&gt; 40 -&gt; 46 -&gt; 50 -&gt; 54 -&gt; 58 -&gt; 62 -&gt; 66 | Speed: 1.3x</t>
+Accuracy: 86% (+1%/Lv) | TP Cost: 22 (+4-6/Lv) -&gt; 66 | Speed: 1.3x</t>
         </is>
       </c>
       <c r="I226" t="inlineStr"/>
@@ -14459,10 +14523,14 @@
       </c>
       <c r="K226" t="inlineStr"/>
       <c r="L226" t="inlineStr"/>
-      <c r="M226" t="inlineStr"/>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
       <c r="N226" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O226" t="inlineStr"/>
@@ -14505,7 +14573,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>Pwr: 240 -&gt; 280 -&gt; 320 -&gt; 360 -&gt; 400 -&gt; 440 -&gt; 480 -&gt; 520 -&gt; 560 -&gt; 600 | Stun: 25%
+          <t>Pwr: 240 (+40/Lv) -&gt; 600 (L10 Max) | Accuracy: 76% (+1%/Lv) | Stun: 25%
 TP Cost: 36 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 -&gt; 66 -&gt; 72 -&gt; 80 -&gt; 88 -&gt; 96 | Speed: 1.5x</t>
         </is>
       </c>
@@ -14520,7 +14588,7 @@
       <c r="M227" t="inlineStr"/>
       <c r="N227" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O227" t="inlineStr"/>
@@ -14934,7 +15002,7 @@
       <c r="H234" t="inlineStr">
         <is>
           <t>Pwr: 100 -&gt; 130 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 280 -&gt; 320 -&gt; 370 -&gt; 420 -&gt; 480 (L10)
-TP Cost: 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 -&gt; 54 -&gt; 58 -&gt; 62 -&gt; 66 | Speed: 0.85x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 30 (+4/Lv) -&gt; 66 | Speed: 0.85x</t>
         </is>
       </c>
       <c r="I234" t="inlineStr"/>
@@ -14945,10 +15013,14 @@
       </c>
       <c r="K234" t="inlineStr"/>
       <c r="L234" t="inlineStr"/>
-      <c r="M234" t="inlineStr"/>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
       <c r="N234" t="inlineStr">
         <is>
-          <t>Accuracy, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O234" t="inlineStr"/>
@@ -14991,8 +15063,8 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>Pwr: 360 -&gt; 400 -&gt; 440 -&gt; 480 -&gt; 520 -&gt; 560 -&gt; 600 -&gt; 640 -&gt; 690 -&gt; 740 (L10)
-Instakill: 12% | TP Cost: 32 -&gt; 35 -&gt; 38 -&gt; 41 -&gt; 44 -&gt; 47 -&gt; 50 -&gt; 52 -&gt; 54 -&gt; 56</t>
+          <t>Pwr: 360 (+40-50/Lv) -&gt; 740 | Accuracy: 76% (+1%/Lv) | Instakill: 12%
+TP Cost: 32 -&gt; 35 -&gt; 38 -&gt; 41 -&gt; 44 -&gt; 47 -&gt; 50 -&gt; 52 -&gt; 54 -&gt; 56 | Speed: 1.2x</t>
         </is>
       </c>
       <c r="I235" t="inlineStr"/>
@@ -15003,10 +15075,14 @@
       </c>
       <c r="K235" t="inlineStr"/>
       <c r="L235" t="inlineStr"/>
-      <c r="M235" t="inlineStr"/>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Pwr</t>
+        </is>
+      </c>
       <c r="N235" t="inlineStr">
         <is>
-          <t>Accuracy, Speed, Chant</t>
+          <t>Chant</t>
         </is>
       </c>
       <c r="O235" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: qoL roadmap, line 1 of skills for the battle bar, enemy attack
qoL roadmap, line 1 of skills for the battle bar, enemy attack chances

- docs/QOL_ROADMAP.md: every pack with real counts, what is open, the
screens still to look at and the order of work for calling QoL done. -
Line 1 of techniques and spells (the battle bar, no level shown): damage
as one word on the scale chosen chosen by the average of the real
values, ailment chance as the shortest true figure (25%, 30%+, 20-50%).
Skills with effects that are not understood stay as written. - Enemy
attacks (also summon abilities): exact ailment chance on the data line
of 858 of 2,375 entries; prose and jokes checked identical. -
EnemyAttackHelper rewrites all 2,375 entries byte for byte. - Spec
amended with the rules of 2026-10-04.

72 tests.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_skill_text.xlsx
+++ b/mod_project/data_tables/qol_skill_text.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P331"/>
+  <dimension ref="A1:Q331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -449,6 +449,7 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="84" customWidth="1" min="15" max="15"/>
     <col width="86" customWidth="1" min="16" max="16"/>
+    <col width="90" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,6 +531,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Previous_Mod_LvUp</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Line1_Notes</t>
         </is>
       </c>
     </row>
@@ -595,6 +601,7 @@
 TP Cost: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -658,6 +665,7 @@
 TP Cost: 3 -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 11</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -725,6 +733,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -758,7 +767,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Short-range skill. Powerful strike to one enemy.</t>
+          <t>Short-range skill. Major strike to one enemy.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -792,6 +801,7 @@
 TP Cost: 5 -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -859,6 +869,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -930,6 +941,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1001,6 +1013,7 @@
 ATK: -11% -&gt; -25% (-3.5%/Lv) | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1034,7 +1047,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Shield skill. Deal bash damage to one enemy. May stun.</t>
+          <t>Shield skill. Deal minor bash damage to one enemy. May stun (30%+).</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1072,6 +1085,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 | Requires equipped shield</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1105,7 +1119,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Katana skill. Deal bash damage to one enemy. May paralyze.</t>
+          <t>Katana skill. Deal moderate bash damage to one enemy. May paralyze (20-50%).</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1143,6 +1157,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1218,6 +1233,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1251,7 +1267,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Katana skill. Deal slash damage to an enemy row. May instakill.</t>
+          <t>Katana skill. Deal slash damage to an enemy row. May instakill (10%+).</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1283,6 +1299,11 @@
         <is>
           <t>ATK: 115% -&gt; 175% (+15%/Lv) | Instakill: 10% -&gt; 25% (+3.75%/Lv)
 TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 136</t>
         </is>
       </c>
     </row>
@@ -1348,6 +1369,11 @@
 TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 | Bypasses enemy armor</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 69</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1381,7 +1407,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Katana skill. Deal slash damage to an enemy row.</t>
+          <t>Katana skill. Deal minor slash damage to an enemy row.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1415,6 +1441,7 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1482,6 +1509,11 @@
 TP Cost: 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 | Target must be living (not undead)</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 31, 87, 90</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1515,7 +1547,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Short-range skill. Attack one enemy to regain HP.</t>
+          <t>Short-range skill. Deal minor damage to one enemy to regain HP.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1549,6 +1581,7 @@
 HP Absorb: 20% -&gt; 30% -&gt; 40% -&gt; 50% -&gt; 60% | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1582,7 +1615,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Short-range skill. Attack one enemy to regain TP.</t>
+          <t>Short-range skill. Deal minor damage to one enemy to regain TP.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1616,6 +1649,7 @@
 TP Absorb: 5% -&gt; 8% -&gt; 11% -&gt; 14% -&gt; 18% | TP Cost: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1649,7 +1683,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Short-range skill. Deal mid-range water damage to one enemy. May freeze.</t>
+          <t>Short-range skill. Deal severe mid-range water damage to one enemy. May freeze.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1683,6 +1717,11 @@
 TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>chance left out: the sentence would be 88 characters</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1716,7 +1755,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Axe skill. Deal earth damage to one enemy. May petrify.</t>
+          <t>Axe skill. Deal severe earth damage to one enemy. May petrify (20-35%).</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1750,6 +1789,7 @@
 TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1821,6 +1861,11 @@
 TP Cost: 16 -&gt; 19 -&gt; 22 -&gt; 25 -&gt; 28 | Hits 2 sequential turn targets</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>damage is major but the sentence would be 90 characters</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1888,6 +1933,7 @@
 TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 20 -&gt; 24 | Requires 1H weapon &amp; shield</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1955,6 +2001,7 @@
 TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22 | May break on repeat blocks</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2020,6 +2067,11 @@
         <is>
           <t>ATK: 140% -&gt; 155% -&gt; 170% -&gt; 185% -&gt; 200% (L1-5) | Unholy Bonus: 1.50x
 TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 88</t>
         </is>
       </c>
     </row>
@@ -2089,6 +2141,7 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 | Requires shield</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2156,6 +2209,7 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 | Requires shield</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2189,7 +2243,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Short-range skill. Deal lightning damage to an enemy row. May paralyze.</t>
+          <t>Short-range skill. Deal minor lightning damage to an enemy row. May paralyze.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2223,6 +2277,11 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>chance left out: the sentence would be 86 characters</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2256,7 +2315,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Lance skill. Deal wind damage to one enemy. May silence.</t>
+          <t>Lance skill. Deal severe wind damage to one enemy. May silence (20-50%).</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2290,6 +2349,7 @@
 TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2357,6 +2417,11 @@
 TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28 | Heavy Lance bonus: +20% dmg</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 96, 111</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2390,7 +2455,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Sword/lance skill. Pierces through to the back row.</t>
+          <t>Sword/lance skill. Pierces through to the back row for major damage.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2424,6 +2489,7 @@
 TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2495,6 +2561,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 | Applies to next physical action</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2557,6 +2624,7 @@
 TP Cost: 2 -&gt; 3 -&gt; 4 -&gt; 5 -&gt; 6</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2619,6 +2687,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2682,6 +2751,11 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 70</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2745,6 +2819,11 @@
 TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 71</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2812,6 +2891,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2879,6 +2959,7 @@
 TP Cost: 3 -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 11 (L1-5)</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2950,6 +3031,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3013,6 +3095,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3088,6 +3171,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3121,7 +3205,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Short-range skill. Attack one enemy. May cause sleep.</t>
+          <t>Short-range skill. Deal moderate damage to one enemy. May cause sleep (20-50%).</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3155,6 +3239,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3188,7 +3273,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Short-range skill. Attack one enemy. May silence.</t>
+          <t>Short-range skill. Deal moderate damage to one enemy. May silence (20-50%).</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3222,6 +3307,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3255,7 +3341,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Short-range skill. Attack one enemy. May stun.</t>
+          <t>Short-range skill. Deal moderate damage to one enemy. May stun (20-50%).</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3289,6 +3375,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3354,6 +3441,11 @@
         <is>
           <t>Hits: 2 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 | ATK: 65% -&gt; 85% per hit (+5%/Lv)
 TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 25</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 93, 125, 136</t>
         </is>
       </c>
     </row>
@@ -3419,6 +3511,11 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 72</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3490,6 +3587,11 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 73</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3523,7 +3625,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Bow/gun skill. Attack one enemy. May poison.</t>
+          <t>Bow/gun skill. Deal moderate damage to one enemy. May poison (20-50%).</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3557,6 +3659,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3590,7 +3693,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Bow skill. Deal stab damage to one enemy. May freeze.</t>
+          <t>Bow skill. Deal moderate stab damage to one enemy. May freeze (20-50%).</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3624,6 +3727,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3657,7 +3761,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Bow skill. Deal stab damage to one enemy. May paralyze.</t>
+          <t>Bow skill. Deal moderate stab damage to one enemy. May paralyze (20-50%).</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -3691,6 +3795,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3724,7 +3829,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Bow skill. Deal stab damage to one enemy. May slow.</t>
+          <t>Bow skill. Deal moderate stab damage to one enemy. May slow (20-50%).</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3758,6 +3863,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3791,7 +3897,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Bow skill. Shoot a barrage of arrows that rains upon all enemies.</t>
+          <t>Bow skill. Shoot a barrage of arrows that rains minor damage upon all enemies.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3821,6 +3927,7 @@
 TP Cost: 16 -&gt; 19 -&gt; 22 -&gt; 25 -&gt; 28</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3892,6 +3999,11 @@
 Duration: 2 -&gt; 3 turns | TP Cost: 20 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 36</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 146, 147</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3959,6 +4071,11 @@
 TP Cost: 18 -&gt; 22 -&gt; 26 -&gt; 30 -&gt; 34 | Hits both front and back target</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 31</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4021,6 +4138,11 @@
       </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 79, 168</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4054,7 +4176,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Deal bash damage to one enemy. May stun.</t>
+          <t>Deal major bash damage to one enemy. May stun (10%+).</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4092,6 +4214,7 @@
 TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4154,6 +4277,7 @@
 TP Cost: 5 -&gt; 4 -&gt; 3 -&gt; 2 -&gt; 1 (Max)</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4212,6 +4336,7 @@
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4287,6 +4412,11 @@
 TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 73</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4320,7 +4450,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Mace skill. Decrease the enemy's DEF as you attack.</t>
+          <t>Mace skill. Decrease the enemy's DEF as you deal severe damage.</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4354,6 +4484,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 | Fast turn recovery (0.85x delay)</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4387,7 +4518,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Sword skill. Deal slash damage to all enemies.</t>
+          <t>Sword skill. Deal moderate slash damage to all enemies.</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4421,6 +4552,7 @@
 TP Cost: 36 -&gt; 46 -&gt; 57 -&gt; 68 -&gt; 79 | Action delay: 0.80x -&gt; 0.98x</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4483,6 +4615,7 @@
       </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4546,6 +4679,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4579,7 +4713,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Short-range skill. Perform a powerful lightning strike to one enemy.</t>
+          <t>Short-range skill. Perform a major lightning strike to one enemy.</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -4613,6 +4747,7 @@
 TP Cost: 13 -&gt; 20 -&gt; 28 -&gt; 36 -&gt; 45</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4646,7 +4781,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Tome skill. RES-based bash damage to one enemy. May freeze/silence.</t>
+          <t>Tome skill. RES-based bash damage to one enemy. May freeze/silence (20-50%).</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4671,6 +4806,11 @@
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 47</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4725,6 +4865,7 @@
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4769,6 +4910,7 @@
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4830,6 +4972,7 @@
 TP Cost: 2 -&gt; 4 -&gt; 6 -&gt; 8 -&gt; 10 | Affected by Maid Mastery (+10% cap)</t>
         </is>
       </c>
+      <c r="Q66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4892,6 +5035,7 @@
 Action delay: 0.85x | TP Cost: 0 (Costs no TP to use)</t>
         </is>
       </c>
+      <c r="Q67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4953,6 +5097,7 @@
 Leaves user at 0 TP | Fast recovery</t>
         </is>
       </c>
+      <c r="Q68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5015,6 +5160,7 @@
 Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 | TP Cost: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12</t>
         </is>
       </c>
+      <c r="Q69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5077,6 +5223,7 @@
 TP Cost: 0 | Action delay: 1.00x</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5139,6 +5286,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5201,6 +5349,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5254,6 +5403,7 @@
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5307,6 +5457,7 @@
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5369,6 +5520,7 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5422,6 +5574,7 @@
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5475,6 +5628,7 @@
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5540,6 +5694,11 @@
         <is>
           <t>ATK: 120% -&gt; 180% (+15%/Lv) | Row bash attack
 TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 (L1-5)</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 136</t>
         </is>
       </c>
     </row>
@@ -5596,6 +5755,11 @@
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 95</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5654,6 +5818,11 @@
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 93; chance not stated: the ailments of this sentence have different chances, or one always happens</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5719,6 +5888,11 @@
         <is>
           <t>ATK per hit: 90% -&gt; 110% -&gt; 130% -&gt; 150% -&gt; 180% (L1-5)
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 | Boosted by Trump / High Risk</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 94</t>
         </is>
       </c>
     </row>
@@ -5784,6 +5958,7 @@
 TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 | Action delay: 1.50x (fast)</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5828,6 +6003,7 @@
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5861,7 +6037,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Attack one enemy. May instakill.</t>
+          <t>Deal major damage to one enemy. May instakill (15%+).</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -5895,6 +6071,7 @@
 TP Cost: 16 -&gt; 19 -&gt; 22 -&gt; 25 -&gt; 28 (L1-5)</t>
         </is>
       </c>
+      <c r="Q84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5928,7 +6105,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>50/50 chance of non-elemental damage to each enemy. May stun.</t>
+          <t>50/50 chance of minor non-elemental damage to each enemy. May stun (40-70%).</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -5953,6 +6130,7 @@
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6020,6 +6198,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
         </is>
       </c>
+      <c r="Q86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6064,6 +6243,7 @@
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6118,6 +6298,7 @@
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6151,7 +6332,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage to all enemies with a storm of roses. May poison.</t>
+          <t>Deal moderate non-elemental damage to all enemies with a storm of roses. May poison.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -6176,6 +6357,11 @@
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>chance left out: the sentence would be 93 characters</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6209,7 +6395,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Fan skill. Deal bashing damage to one enemy. May delay enemy turn.</t>
+          <t>Fan skill. Deal severe bashing damage to one enemy. May delay enemy turn.</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -6243,6 +6429,7 @@
 TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6271,7 +6458,7 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Fan skill. With increased ATK, deal long-range damage to one enemy.</t>
+          <t>Fan skill. With increased ATK, deal minor long-range damage to one enemy.</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -6292,6 +6479,7 @@
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6325,7 +6513,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Short-range skill. Pierce through to the back row with stab damage. May slow.</t>
+          <t>Short-range skill. Pierce through to the back row with major stab damage. May slow.</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6350,6 +6538,11 @@
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>chance left out: the sentence would be 92 characters</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6408,6 +6601,11 @@
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 133</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6471,6 +6669,7 @@
 Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 | TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26</t>
         </is>
       </c>
+      <c r="Q94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6515,6 +6714,7 @@
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6577,6 +6777,11 @@
       </c>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 99, 110</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6652,6 +6857,7 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 (L1-5)</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6714,6 +6920,7 @@
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6785,6 +6992,7 @@
 TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 (L1-5)</t>
         </is>
       </c>
+      <c r="Q99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6847,6 +7055,7 @@
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6914,6 +7123,7 @@
 TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 (L1-5)</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6985,6 +7195,7 @@
 TP Cost: 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 (L1-5)</t>
         </is>
       </c>
+      <c r="Q102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7039,6 +7250,7 @@
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7093,6 +7305,7 @@
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7147,6 +7360,7 @@
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7201,6 +7415,7 @@
       <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7255,6 +7470,7 @@
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7309,6 +7525,7 @@
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7363,6 +7580,7 @@
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr"/>
+      <c r="Q109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7417,6 +7635,7 @@
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7471,6 +7690,7 @@
       <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr"/>
+      <c r="Q111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7525,6 +7745,7 @@
       <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr"/>
+      <c r="Q112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7579,6 +7800,7 @@
       <c r="N113" t="inlineStr"/>
       <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr"/>
+      <c r="Q113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7633,6 +7855,7 @@
       <c r="N114" t="inlineStr"/>
       <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr"/>
+      <c r="Q114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7687,6 +7910,7 @@
       <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr"/>
       <c r="P115" t="inlineStr"/>
+      <c r="Q115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7741,6 +7965,7 @@
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr"/>
+      <c r="Q116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -7795,6 +8020,7 @@
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr"/>
       <c r="P117" t="inlineStr"/>
+      <c r="Q117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -7849,6 +8075,7 @@
       <c r="N118" t="inlineStr"/>
       <c r="O118" t="inlineStr"/>
       <c r="P118" t="inlineStr"/>
+      <c r="Q118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -7903,6 +8130,7 @@
       <c r="N119" t="inlineStr"/>
       <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr"/>
+      <c r="Q119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7957,6 +8185,7 @@
       <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8011,6 +8240,7 @@
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8065,6 +8295,7 @@
       <c r="N122" t="inlineStr"/>
       <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8119,6 +8350,7 @@
       <c r="N123" t="inlineStr"/>
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8173,6 +8405,7 @@
       <c r="N124" t="inlineStr"/>
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8227,6 +8460,7 @@
       <c r="N125" t="inlineStr"/>
       <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8281,6 +8515,7 @@
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -8335,6 +8570,7 @@
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8389,6 +8625,7 @@
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8443,6 +8680,7 @@
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr"/>
+      <c r="Q129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8497,6 +8735,7 @@
       <c r="N130" t="inlineStr"/>
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8551,6 +8790,7 @@
       <c r="N131" t="inlineStr"/>
       <c r="O131" t="inlineStr"/>
       <c r="P131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -8605,6 +8845,7 @@
       <c r="N132" t="inlineStr"/>
       <c r="O132" t="inlineStr"/>
       <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -8659,6 +8900,7 @@
       <c r="N133" t="inlineStr"/>
       <c r="O133" t="inlineStr"/>
       <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -8713,6 +8955,7 @@
       <c r="N134" t="inlineStr"/>
       <c r="O134" t="inlineStr"/>
       <c r="P134" t="inlineStr"/>
+      <c r="Q134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -8767,6 +9010,7 @@
       <c r="N135" t="inlineStr"/>
       <c r="O135" t="inlineStr"/>
       <c r="P135" t="inlineStr"/>
+      <c r="Q135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -8821,6 +9065,7 @@
       <c r="N136" t="inlineStr"/>
       <c r="O136" t="inlineStr"/>
       <c r="P136" t="inlineStr"/>
+      <c r="Q136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -8875,6 +9120,7 @@
       <c r="N137" t="inlineStr"/>
       <c r="O137" t="inlineStr"/>
       <c r="P137" t="inlineStr"/>
+      <c r="Q137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -8929,6 +9175,7 @@
       <c r="N138" t="inlineStr"/>
       <c r="O138" t="inlineStr"/>
       <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -8983,6 +9230,7 @@
       <c r="N139" t="inlineStr"/>
       <c r="O139" t="inlineStr"/>
       <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9037,6 +9285,7 @@
       <c r="N140" t="inlineStr"/>
       <c r="O140" t="inlineStr"/>
       <c r="P140" t="inlineStr"/>
+      <c r="Q140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -9091,6 +9340,7 @@
       <c r="N141" t="inlineStr"/>
       <c r="O141" t="inlineStr"/>
       <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -9145,6 +9395,7 @@
       <c r="N142" t="inlineStr"/>
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9199,6 +9450,7 @@
       <c r="N143" t="inlineStr"/>
       <c r="O143" t="inlineStr"/>
       <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9253,6 +9505,7 @@
       <c r="N144" t="inlineStr"/>
       <c r="O144" t="inlineStr"/>
       <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9286,7 +9539,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Deal fire damage to one enemy.</t>
+          <t>Deal moderate fire damage to one enemy.</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -9324,6 +9577,7 @@
 TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -9357,7 +9611,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Deal fire damage to an enemy row.</t>
+          <t>Deal moderate fire damage to an enemy row.</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -9395,6 +9649,7 @@
 TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -9428,7 +9683,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Deal fire damage to all enemies.</t>
+          <t>Deal severe fire damage to all enemies.</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -9466,6 +9721,7 @@
 TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -9529,6 +9785,7 @@
 TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -9562,7 +9819,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Deal water damage to one enemy.</t>
+          <t>Deal moderate water damage to one enemy.</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -9600,6 +9857,7 @@
 TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -9633,7 +9891,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Deal water damage to an enemy row.</t>
+          <t>Deal moderate water damage to an enemy row.</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -9671,6 +9929,7 @@
 TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -9704,7 +9963,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Deal water damage to all enemies.</t>
+          <t>Deal severe water damage to all enemies.</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -9742,6 +10001,7 @@
 TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -9805,6 +10065,7 @@
 TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -9838,7 +10099,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Deal lightning damage to one enemy.</t>
+          <t>Deal moderate lightning damage to one enemy.</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -9876,6 +10137,7 @@
 TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -9909,7 +10171,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Deal lightning damage to an enemy row.</t>
+          <t>Deal moderate lightning damage to an enemy row.</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -9947,6 +10209,7 @@
 TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -9980,7 +10243,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Deal lightning damage to all enemies.</t>
+          <t>Deal severe lightning damage to all enemies.</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -10018,6 +10281,7 @@
 TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -10081,6 +10345,7 @@
 TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10114,7 +10379,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Deal wind damage to one enemy.</t>
+          <t>Deal moderate wind damage to one enemy.</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -10152,6 +10417,7 @@
 TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10185,7 +10451,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Deal wind damage to an enemy row.</t>
+          <t>Deal moderate wind damage to an enemy row.</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -10223,6 +10489,7 @@
 TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -10256,7 +10523,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Deal wind damage to all enemies.</t>
+          <t>Deal severe wind damage to all enemies.</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -10294,6 +10561,7 @@
 TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -10357,6 +10625,7 @@
 TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -10390,7 +10659,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Deal earth damage to one enemy.</t>
+          <t>Deal moderate earth damage to one enemy.</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -10428,6 +10697,7 @@
 TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -10461,7 +10731,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Deal earth damage to an enemy row.</t>
+          <t>Deal moderate earth damage to an enemy row.</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -10499,6 +10769,7 @@
 TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -10532,7 +10803,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Deal earth damage to all enemies.</t>
+          <t>Deal severe earth damage to all enemies.</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -10570,6 +10841,7 @@
 TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -10633,6 +10905,7 @@
 TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -10666,7 +10939,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage to one enemy to regain HP.</t>
+          <t>Deal minor non-elemental damage to one enemy to regain HP.</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -10704,6 +10977,7 @@
 TP Cost: 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -10737,7 +11011,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage to one enemy to regain TP.</t>
+          <t>Deal negligible non-elemental damage to one enemy to regain TP.</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -10775,6 +11049,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 15</t>
         </is>
       </c>
+      <c r="Q166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -10842,6 +11117,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -10875,7 +11151,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Absorb HP from an enemy row.</t>
+          <t>Absorb HP from an enemy row with moderate damage.</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -10913,6 +11189,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 (L1-5)</t>
         </is>
       </c>
+      <c r="Q168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -10946,7 +11223,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Stun one enemy.</t>
+          <t>Stun one enemy (65%+).</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
@@ -10976,6 +11253,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -11009,7 +11287,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Poison all enemies.</t>
+          <t>Poison all enemies (75%+).</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -11039,6 +11317,7 @@
 TP Cost: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5)</t>
         </is>
       </c>
+      <c r="Q170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -11072,7 +11351,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Freeze all enemies.</t>
+          <t>Freeze all enemies (70%+).</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -11102,6 +11381,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -11135,7 +11415,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Paralyze all enemies.</t>
+          <t>Paralyze all enemies (65%+).</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -11165,6 +11445,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -11198,7 +11479,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Put an enemy row to sleep.</t>
+          <t>Put an enemy row to sleep (65%+).</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -11228,6 +11509,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -11261,7 +11543,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Silence all enemies.</t>
+          <t>Silence all enemies (70%+).</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -11291,6 +11573,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -11324,7 +11607,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Petrify an enemy row.</t>
+          <t>Petrify an enemy row (70%+).</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -11354,6 +11637,7 @@
 TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22</t>
         </is>
       </c>
+      <c r="Q175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -11387,7 +11671,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Instakill one enemy.</t>
+          <t>Instakill one enemy (50%+).</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -11417,6 +11701,7 @@
 TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28</t>
         </is>
       </c>
+      <c r="Q176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -11450,7 +11735,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Slow an enemy row.</t>
+          <t>Slow an enemy row (50-68%).</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -11480,6 +11765,7 @@
 TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 (L1-5)</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -11513,7 +11799,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Stun an enemy row.</t>
+          <t>Stun an enemy row (54-70%).</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -11543,6 +11829,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -11597,6 +11884,7 @@
       <c r="N179" t="inlineStr"/>
       <c r="O179" t="inlineStr"/>
       <c r="P179" t="inlineStr"/>
+      <c r="Q179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -11659,6 +11947,11 @@
       </c>
       <c r="O180" t="inlineStr"/>
       <c r="P180" t="inlineStr"/>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 88</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -11722,6 +12015,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -11785,6 +12079,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -11848,6 +12143,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -11911,6 +12207,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -11974,6 +12271,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -12041,6 +12339,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -12108,6 +12407,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -12175,6 +12475,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
         </is>
       </c>
+      <c r="Q188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -12246,6 +12547,7 @@
 TP Cost: 3 -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -12317,6 +12619,7 @@
 TP Cost: 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 21 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 -&gt; 46  (Lv1 to Max)</t>
         </is>
       </c>
+      <c r="Q190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -12378,6 +12681,7 @@
 TP Cost: 35 -&gt; 30 -&gt; 25 -&gt; 20 -&gt; 16 (L1-5)</t>
         </is>
       </c>
+      <c r="Q191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -12445,6 +12749,7 @@
 TP Cost: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 (L1-7)</t>
         </is>
       </c>
+      <c r="Q192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -12512,6 +12817,7 @@
 TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 (L1-7)</t>
         </is>
       </c>
+      <c r="Q193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -12575,6 +12881,7 @@
 Chant time decreases per level | TP Cost: 18 -&gt; 22 -&gt; 26 -&gt; 30 -&gt; 35</t>
         </is>
       </c>
+      <c r="Q194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -12642,6 +12949,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -12709,6 +13017,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -12776,6 +13085,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
         </is>
       </c>
+      <c r="Q197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -12843,6 +13153,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
         </is>
       </c>
+      <c r="Q198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -12910,6 +13221,7 @@
 Chant time decreases per level | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -12977,6 +13289,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22</t>
         </is>
       </c>
+      <c r="Q200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13044,6 +13357,7 @@
 TP Cost: 7 -&gt; 10 -&gt; 13 -&gt; 16 -&gt; 20 -&gt; 24 -&gt; 28 (L1-7)</t>
         </is>
       </c>
+      <c r="Q201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -13107,6 +13421,7 @@
 Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-5) | TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22</t>
         </is>
       </c>
+      <c r="Q202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -13170,6 +13485,7 @@
 TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
         </is>
       </c>
+      <c r="Q203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -13228,6 +13544,7 @@
       </c>
       <c r="O204" t="inlineStr"/>
       <c r="P204" t="inlineStr"/>
+      <c r="Q204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -13289,6 +13606,7 @@
 TP Cost: 4 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 4</t>
         </is>
       </c>
+      <c r="Q205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -13350,6 +13668,7 @@
 Works identical to an Emergency Exit item</t>
         </is>
       </c>
+      <c r="Q206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -13382,7 +13701,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>Put an enemy to sleep.</t>
+          <t>Put an enemy to sleep (70-82%).</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -13412,6 +13731,7 @@
 TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
+      <c r="Q207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -13460,6 +13780,7 @@
       <c r="N208" t="inlineStr"/>
       <c r="O208" t="inlineStr"/>
       <c r="P208" t="inlineStr"/>
+      <c r="Q208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -13513,6 +13834,7 @@
       <c r="N209" t="inlineStr"/>
       <c r="O209" t="inlineStr"/>
       <c r="P209" t="inlineStr"/>
+      <c r="Q209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -13566,6 +13888,7 @@
       <c r="N210" t="inlineStr"/>
       <c r="O210" t="inlineStr"/>
       <c r="P210" t="inlineStr"/>
+      <c r="Q210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -13619,6 +13942,7 @@
       <c r="N211" t="inlineStr"/>
       <c r="O211" t="inlineStr"/>
       <c r="P211" t="inlineStr"/>
+      <c r="Q211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -13672,6 +13996,7 @@
       <c r="N212" t="inlineStr"/>
       <c r="O212" t="inlineStr"/>
       <c r="P212" t="inlineStr"/>
+      <c r="Q212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -13734,6 +14059,7 @@
 Chant Time: 2 turns -&gt; 1 turn | TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
         </is>
       </c>
+      <c r="Q213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -13796,6 +14122,7 @@
 Chant Time: 2 turns -&gt; 1 turn | TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22</t>
         </is>
       </c>
+      <c r="Q214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -13858,6 +14185,7 @@
 TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22</t>
         </is>
       </c>
+      <c r="Q215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -13920,6 +14248,7 @@
 TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
+      <c r="Q216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -13973,6 +14302,7 @@
       <c r="N217" t="inlineStr"/>
       <c r="O217" t="inlineStr"/>
       <c r="P217" t="inlineStr"/>
+      <c r="Q217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -14031,6 +14361,7 @@
       </c>
       <c r="O218" t="inlineStr"/>
       <c r="P218" t="inlineStr"/>
+      <c r="Q218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -14085,6 +14416,7 @@
       <c r="N219" t="inlineStr"/>
       <c r="O219" t="inlineStr"/>
       <c r="P219" t="inlineStr"/>
+      <c r="Q219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -14139,6 +14471,7 @@
       <c r="N220" t="inlineStr"/>
       <c r="O220" t="inlineStr"/>
       <c r="P220" t="inlineStr"/>
+      <c r="Q220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -14205,6 +14538,7 @@
       </c>
       <c r="O221" t="inlineStr"/>
       <c r="P221" t="inlineStr"/>
+      <c r="Q221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -14275,6 +14609,7 @@
       </c>
       <c r="O222" t="inlineStr"/>
       <c r="P222" t="inlineStr"/>
+      <c r="Q222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -14341,6 +14676,7 @@
       </c>
       <c r="O223" t="inlineStr"/>
       <c r="P223" t="inlineStr"/>
+      <c r="Q223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -14407,6 +14743,7 @@
       </c>
       <c r="O224" t="inlineStr"/>
       <c r="P224" t="inlineStr"/>
+      <c r="Q224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -14473,6 +14810,7 @@
       </c>
       <c r="O225" t="inlineStr"/>
       <c r="P225" t="inlineStr"/>
+      <c r="Q225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -14506,7 +14844,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage to an enemy row.</t>
+          <t>Deal severe non-elemental damage to an enemy row.</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -14535,6 +14873,7 @@
       </c>
       <c r="O226" t="inlineStr"/>
       <c r="P226" t="inlineStr"/>
+      <c r="Q226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -14568,7 +14907,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage to all enemies. May stun.</t>
+          <t>Deal major non-elemental damage to all enemies. May stun (25%).</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -14593,6 +14932,7 @@
       </c>
       <c r="O227" t="inlineStr"/>
       <c r="P227" t="inlineStr"/>
+      <c r="Q227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -14660,6 +15000,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 14 -&gt; 18 -&gt; 22 -&gt; 26 -&gt; 30</t>
         </is>
       </c>
+      <c r="Q228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -14727,6 +15068,7 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 14 -&gt; 18 -&gt; 22 -&gt; 26 -&gt; 30</t>
         </is>
       </c>
+      <c r="Q229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -14781,6 +15123,7 @@
       <c r="N230" t="inlineStr"/>
       <c r="O230" t="inlineStr"/>
       <c r="P230" t="inlineStr"/>
+      <c r="Q230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -14835,6 +15178,7 @@
       <c r="N231" t="inlineStr"/>
       <c r="O231" t="inlineStr"/>
       <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -14897,6 +15241,7 @@
       <c r="N232" t="inlineStr"/>
       <c r="O232" t="inlineStr"/>
       <c r="P232" t="inlineStr"/>
+      <c r="Q232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -14963,6 +15308,7 @@
       </c>
       <c r="O233" t="inlineStr"/>
       <c r="P233" t="inlineStr"/>
+      <c r="Q233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -15025,6 +15371,11 @@
       </c>
       <c r="O234" t="inlineStr"/>
       <c r="P234" t="inlineStr"/>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 47</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -15058,7 +15409,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Deal enormous damage to one enemy that possesses life. Low chance of instakill.</t>
+          <t>Deal enormous damage to one enemy that possesses life. Low chance of instakill (12%).</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -15087,6 +15438,11 @@
       </c>
       <c r="O235" t="inlineStr"/>
       <c r="P235" t="inlineStr"/>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>no damage word: carries effects that are not understood: 87</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -15149,6 +15505,7 @@
       <c r="N236" t="inlineStr"/>
       <c r="O236" t="inlineStr"/>
       <c r="P236" t="inlineStr"/>
+      <c r="Q236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -15203,6 +15560,7 @@
       <c r="N237" t="inlineStr"/>
       <c r="O237" t="inlineStr"/>
       <c r="P237" t="inlineStr"/>
+      <c r="Q237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -15257,6 +15615,7 @@
       <c r="N238" t="inlineStr"/>
       <c r="O238" t="inlineStr"/>
       <c r="P238" t="inlineStr"/>
+      <c r="Q238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -15311,6 +15670,7 @@
       <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr"/>
       <c r="P239" t="inlineStr"/>
+      <c r="Q239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -15365,6 +15725,7 @@
       <c r="N240" t="inlineStr"/>
       <c r="O240" t="inlineStr"/>
       <c r="P240" t="inlineStr"/>
+      <c r="Q240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -15419,6 +15780,7 @@
       <c r="N241" t="inlineStr"/>
       <c r="O241" t="inlineStr"/>
       <c r="P241" t="inlineStr"/>
+      <c r="Q241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -15482,6 +15844,7 @@
 Heroine: Melvy</t>
         </is>
       </c>
+      <c r="Q242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -15543,6 +15906,7 @@
 Scales off weapon base ATK (not total character ATK)</t>
         </is>
       </c>
+      <c r="Q243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -15604,6 +15968,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -15665,6 +16030,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -15726,6 +16092,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -15787,6 +16154,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -15848,6 +16216,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -15909,6 +16278,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -15970,6 +16340,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -16031,6 +16402,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -16092,6 +16464,7 @@
 Scales off weapon base ATK</t>
         </is>
       </c>
+      <c r="Q252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -16153,6 +16526,7 @@
 Universal weapon scaling</t>
         </is>
       </c>
+      <c r="Q253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -16214,6 +16588,7 @@
 Applies to all offensive spell damage</t>
         </is>
       </c>
+      <c r="Q254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -16283,6 +16658,7 @@
 Also raises baseline healing cap on Heal and Circle Heal</t>
         </is>
       </c>
+      <c r="Q255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -16344,6 +16720,7 @@
 Triggers at start of user's action in combat</t>
         </is>
       </c>
+      <c r="Q256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -16405,6 +16782,7 @@
 Triggers at start of user's action in combat</t>
         </is>
       </c>
+      <c r="Q257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -16466,6 +16844,7 @@
 Active on user turn in battle</t>
         </is>
       </c>
+      <c r="Q258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -16527,6 +16906,7 @@
 Triggers on user turn in combat</t>
         </is>
       </c>
+      <c r="Q259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -16588,6 +16968,7 @@
 Applies to Fire, Water, Lightning, Wind, and Earth</t>
         </is>
       </c>
+      <c r="Q260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -16649,6 +17030,7 @@
 Note: Short-range retaliations will trigger enemy Dark Aura</t>
         </is>
       </c>
+      <c r="Q261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -16710,6 +17092,7 @@
 Nullifies incoming attack and strikes back</t>
         </is>
       </c>
+      <c r="Q262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -16771,6 +17154,7 @@
 Can stack with Triple Attack (up to 5 strikes total)</t>
         </is>
       </c>
+      <c r="Q263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -16832,6 +17216,7 @@
 Stacks with Double Attack</t>
         </is>
       </c>
+      <c r="Q264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -16884,6 +17269,7 @@
       <c r="N265" t="inlineStr"/>
       <c r="O265" t="inlineStr"/>
       <c r="P265" t="inlineStr"/>
+      <c r="Q265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -16936,6 +17322,7 @@
       <c r="N266" t="inlineStr"/>
       <c r="O266" t="inlineStr"/>
       <c r="P266" t="inlineStr"/>
+      <c r="Q266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -16997,6 +17384,7 @@
 Prevents death when hit by lethal blows</t>
         </is>
       </c>
+      <c r="Q267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -17058,6 +17446,7 @@
 Halves incoming damage when triggered</t>
         </is>
       </c>
+      <c r="Q268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -17119,6 +17508,7 @@
 Main hand weapon deals 100% ATK</t>
         </is>
       </c>
+      <c r="Q269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -17171,6 +17561,7 @@
       <c r="N270" t="inlineStr"/>
       <c r="O270" t="inlineStr"/>
       <c r="P270" t="inlineStr"/>
+      <c r="Q270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -17223,6 +17614,7 @@
       <c r="N271" t="inlineStr"/>
       <c r="O271" t="inlineStr"/>
       <c r="P271" t="inlineStr"/>
+      <c r="Q271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -17275,6 +17667,7 @@
       <c r="N272" t="inlineStr"/>
       <c r="O272" t="inlineStr"/>
       <c r="P272" t="inlineStr"/>
+      <c r="Q272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -17327,6 +17720,7 @@
       <c r="N273" t="inlineStr"/>
       <c r="O273" t="inlineStr"/>
       <c r="P273" t="inlineStr"/>
+      <c r="Q273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -17379,6 +17773,7 @@
       <c r="N274" t="inlineStr"/>
       <c r="O274" t="inlineStr"/>
       <c r="P274" t="inlineStr"/>
+      <c r="Q274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -17431,6 +17826,7 @@
       <c r="N275" t="inlineStr"/>
       <c r="O275" t="inlineStr"/>
       <c r="P275" t="inlineStr"/>
+      <c r="Q275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -17483,6 +17879,7 @@
       <c r="N276" t="inlineStr"/>
       <c r="O276" t="inlineStr"/>
       <c r="P276" t="inlineStr"/>
+      <c r="Q276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -17527,6 +17924,7 @@
       <c r="N277" t="inlineStr"/>
       <c r="O277" t="inlineStr"/>
       <c r="P277" t="inlineStr"/>
+      <c r="Q277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -17571,6 +17969,7 @@
       <c r="N278" t="inlineStr"/>
       <c r="O278" t="inlineStr"/>
       <c r="P278" t="inlineStr"/>
+      <c r="Q278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -17623,6 +18022,7 @@
       <c r="N279" t="inlineStr"/>
       <c r="O279" t="inlineStr"/>
       <c r="P279" t="inlineStr"/>
+      <c r="Q279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -17684,6 +18084,7 @@
 Completely negates incoming physical attacks when triggered</t>
         </is>
       </c>
+      <c r="Q280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -17749,6 +18150,7 @@
 Triggers automatically at start of user's combat turn</t>
         </is>
       </c>
+      <c r="Q281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -17810,6 +18212,7 @@
 Immediate combat stat trigger</t>
         </is>
       </c>
+      <c r="Q282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -17870,6 +18273,7 @@
           <t>Interruption Resist: +20% -&gt; +50% (+7.5%/Lv) | 80% Crit Interrupt Res at Lv 5</t>
         </is>
       </c>
+      <c r="Q283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -17931,6 +18335,7 @@
 Accelerates offensive and healing magic activation</t>
         </is>
       </c>
+      <c r="Q284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -17992,6 +18397,7 @@
 Lowers cost of all techniques and spells</t>
         </is>
       </c>
+      <c r="Q285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -18053,6 +18459,7 @@
 Significantly reduces spell evasion by high RES targets</t>
         </is>
       </c>
+      <c r="Q286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -18114,6 +18521,7 @@
 Protects party from surprise enemy encounters</t>
         </is>
       </c>
+      <c r="Q287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -18175,6 +18583,7 @@
 Grants free initial turn before enemies act</t>
         </is>
       </c>
+      <c r="Q288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -18236,6 +18645,7 @@
 Does not apply to scripted boss battles</t>
         </is>
       </c>
+      <c r="Q289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -18297,6 +18707,7 @@
 Boosts party equipment and material acquisition</t>
         </is>
       </c>
+      <c r="Q290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -18358,6 +18769,7 @@
 Earn bonus currency after every battle</t>
         </is>
       </c>
+      <c r="Q291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -18419,6 +18831,7 @@
 Finds consumables and crafting materials while walking</t>
         </is>
       </c>
+      <c r="Q292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -18488,6 +18901,7 @@
 Restores whole party after combat conclusion</t>
         </is>
       </c>
+      <c r="Q293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -18549,6 +18963,7 @@
 Item is not consumed from inventory when triggered</t>
         </is>
       </c>
+      <c r="Q294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -18610,6 +19025,7 @@
 Applies to all consumable recovery items used in combat</t>
         </is>
       </c>
+      <c r="Q295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -18671,6 +19087,7 @@
 Allows maintaining 2 active Bard songs at once</t>
         </is>
       </c>
+      <c r="Q296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -18732,6 +19149,7 @@
 Allows maintaining 2 active Dancer dances at once</t>
         </is>
       </c>
+      <c r="Q297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -18793,6 +19211,7 @@
 Maintains 2 active summoned dolls simultaneously</t>
         </is>
       </c>
+      <c r="Q298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -18854,6 +19273,7 @@
 Levels: L1-5</t>
         </is>
       </c>
+      <c r="Q299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -18915,6 +19335,7 @@
 Empowers First Aid, Cook, and Clean</t>
         </is>
       </c>
+      <c r="Q300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -18976,6 +19397,7 @@
 Empowers Bard songs and regeneration rates</t>
         </is>
       </c>
+      <c r="Q301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -19037,6 +19459,7 @@
 Empowers Dancer dances and status effects</t>
         </is>
       </c>
+      <c r="Q302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -19098,6 +19521,7 @@
 Increases damage, healing, and durability of summoned dolls</t>
         </is>
       </c>
+      <c r="Q303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -19159,6 +19583,7 @@
 Normal attack trigger</t>
         </is>
       </c>
+      <c r="Q304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -19220,6 +19645,7 @@
 Accelerates Bard song activation</t>
         </is>
       </c>
+      <c r="Q305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -19281,6 +19707,7 @@
 Lowers gold cost for item purchases and item identification</t>
         </is>
       </c>
+      <c r="Q306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -19342,6 +19769,7 @@
 Enemy skips turn when mesmerized</t>
         </is>
       </c>
+      <c r="Q307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -19395,6 +19823,7 @@
 Fixed passive (Level 1)</t>
         </is>
       </c>
+      <c r="Q308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -19448,6 +19877,7 @@
 Fixed passive (Level 1)</t>
         </is>
       </c>
+      <c r="Q309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -19492,6 +19922,7 @@
       <c r="N310" t="inlineStr"/>
       <c r="O310" t="inlineStr"/>
       <c r="P310" t="inlineStr"/>
+      <c r="Q310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -19536,6 +19967,7 @@
       <c r="N311" t="inlineStr"/>
       <c r="O311" t="inlineStr"/>
       <c r="P311" t="inlineStr"/>
+      <c r="Q311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -19589,6 +20021,7 @@
 Spell criticals deal 1.50x normal magic damage</t>
         </is>
       </c>
+      <c r="Q312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -19642,6 +20075,7 @@
 Fixed passive (Level 1)</t>
         </is>
       </c>
+      <c r="Q313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -19693,6 +20127,7 @@
         </is>
       </c>
       <c r="P314" t="inlineStr"/>
+      <c r="Q314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -19744,6 +20179,7 @@
         </is>
       </c>
       <c r="P315" t="inlineStr"/>
+      <c r="Q315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -19795,6 +20231,7 @@
         </is>
       </c>
       <c r="P316" t="inlineStr"/>
+      <c r="Q316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -19846,6 +20283,7 @@
         </is>
       </c>
       <c r="P317" t="inlineStr"/>
+      <c r="Q317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -19897,6 +20335,7 @@
         </is>
       </c>
       <c r="P318" t="inlineStr"/>
+      <c r="Q318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -19948,6 +20387,7 @@
         </is>
       </c>
       <c r="P319" t="inlineStr"/>
+      <c r="Q319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -19999,6 +20439,7 @@
         </is>
       </c>
       <c r="P320" t="inlineStr"/>
+      <c r="Q320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -20050,6 +20491,7 @@
         </is>
       </c>
       <c r="P321" t="inlineStr"/>
+      <c r="Q321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -20101,6 +20543,7 @@
         </is>
       </c>
       <c r="P322" t="inlineStr"/>
+      <c r="Q322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -20152,6 +20595,7 @@
         </is>
       </c>
       <c r="P323" t="inlineStr"/>
+      <c r="Q323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -20203,6 +20647,7 @@
         </is>
       </c>
       <c r="P324" t="inlineStr"/>
+      <c r="Q324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -20254,6 +20699,7 @@
         </is>
       </c>
       <c r="P325" t="inlineStr"/>
+      <c r="Q325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -20305,6 +20751,7 @@
         </is>
       </c>
       <c r="P326" t="inlineStr"/>
+      <c r="Q326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -20356,6 +20803,7 @@
         </is>
       </c>
       <c r="P327" t="inlineStr"/>
+      <c r="Q327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -20407,6 +20855,7 @@
         </is>
       </c>
       <c r="P328" t="inlineStr"/>
+      <c r="Q328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -20458,6 +20907,7 @@
         </is>
       </c>
       <c r="P329" t="inlineStr"/>
+      <c r="Q329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -20509,6 +20959,7 @@
         </is>
       </c>
       <c r="P330" t="inlineStr"/>
+      <c r="Q330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -20560,6 +21011,7 @@
         </is>
       </c>
       <c r="P331" t="inlineStr"/>
+      <c r="Q331" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20714,7 +21166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -20796,34 +21248,58 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Notation</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ATK: 125% -&gt; 134 -&gt; ... -&gt; 200%  |  ATK: 130% (+8%/Lv) -&gt; 202% (L10 Max)  |  Speed: 0.8x -&gt; 0.9x</t>
+          <t>The line shown in battle, where the level is unknown. One word for damage, chosen from the average of the real values (negligible below 80%, minor, moderate, major, severe; tremendous beyond the scale), and the ailment chance as (25%) when it never changes, (30%+) when it rises by 10 points or less, (20-50%) otherwise. No tilde: the game font has none. The build rejects what the binary does not give.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Never</t>
+          <t>Line1_Notes</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Averages such as "(avg +3.33%/Lv)". A step is written only when it is the same at every level.</t>
+          <t>Why a skill got no word: it carries an effect that is not understood, or the sentence would not fit.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Notation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ATK: 125% -&gt; 134 -&gt; ... -&gt; 200%  |  ATK: 130% (+8%/Lv) -&gt; 202% (L10 Max)  |  Speed: 0.8x -&gt; 0.9x</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Averages such as "(avg +3.33%/Lv)". A step is written only when it is the same at every level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Previous_Mod_*</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Wording of the earlier mod, for reference only. Its numbers were not taken from the binary.</t>
         </is>

</xml_diff>

<commit_message>
feat: show every value; items as original +
show every value; items as original + (data); enemy attacks second pass

From the answers to the roadmap's open questions: - Skill boxes show
values that never change with the level too. - Line 1 says the value for
buffs, heals and passives (202 sentences). - A chance of 100% is written
as 100%. - Where the original text and the data disagree the data wins:
11 enemy attack descriptions corrected (5 figures, 6 times "defense"
where the data lowers physical attack), keeping the rest of the
sentence. - Items: the original sentence plus what the item does (165
items).

Roadmap step 4: exact effects on the data line of 1,456 enemy attacks.

Found: CommandData.pck is the game's own table of effect names by id
(317 names). It confirms the decoded effects and names effect 73 "Damage
xn" (Spiral Arrow, Holy Gavel).

93 tests.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_skill_text.xlsx
+++ b/mod_project/data_tables/qol_skill_text.xlsx
@@ -443,7 +443,7 @@
     <col width="87" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="47" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
@@ -699,7 +699,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Raise the party's ATK.</t>
+          <t>Raise the party's ATK (8%+).</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Increase own ATK at the price of lowering own DEF.</t>
+          <t>Increase own ATK at the price of lowering own DEF (ATK 20-50%, DEF 11-25%).</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Increase own DEF at the price of lowering own ATK.</t>
+          <t>Increase own DEF at the price of lowering own ATK (DEF 20-50%, ATK 11-25%).</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1225,7 +1225,11 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 114 characters</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1265,7 +1269,7 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>ATK: 80% -&gt; 83 -&gt; 86 -&gt; 89 -&gt; 91 -&gt; 94 -&gt; 97 -&gt; 100 -&gt; 105 -&gt; 110% (L10)
-Instakill: 10% (+1-2%/Lv) -&gt; 20% | TP Cost: 38 (+4/Lv) -&gt; 74 | Speed: 0.65x -&gt; 0.75x</t>
+Instakill: 10% (+1-2%/Lv) -&gt; 20% | Power decrease: 10% | TP Cost: 38 (+4/Lv) -&gt; 74</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1281,7 +1285,11 @@
           <t>Instakill</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
           <t>Katana skill. Deal slash damage to an enemy row. May instakill.</t>
@@ -1465,7 +1473,7 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>ATK: 118% -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 146 -&gt; 152 -&gt; 158% (L10)
-TP Cost: 36 -&gt; 38 -&gt; 40 -&gt; 43 -&gt; 46 -&gt; 49 -&gt; 52 -&gt; 55 -&gt; 58 -&gt; 61</t>
+Critical rate: 10% | TP Cost: 36 (+2-3/Lv) -&gt; 61 | Speed: 0.7x -&gt; 0.8x</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1476,12 +1484,12 @@
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>Katana skill. Strike 3 times against one living enemy.</t>
@@ -1669,7 +1677,7 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>ATK: 130% -&gt; 144 -&gt; 157 -&gt; 170 -&gt; 182 -&gt; 194 -&gt; 204 -&gt; 212 -&gt; 220 -&gt; 228% (L10)
-Freeze: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 9 (+3/Lv) -&gt; 36 | Speed: 0.75x -&gt; 0.85x</t>
+Freeze: 20% (+3-4%/Lv) -&gt; 50% | Accuracy: +14% | TP Cost: 9 (+3/Lv) -&gt; 36</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1685,7 +1693,11 @@
           <t>Freeze</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
       <c r="O18" t="inlineStr">
         <is>
           <t>Short-range strike dealing mid-range water damage. May freeze.</t>
@@ -1740,8 +1752,8 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ATK: 135% -&gt; 149 -&gt; 163 -&gt; 176 -&gt; 189 -&gt; 201 -&gt; 213 -&gt; 225 -&gt; 236 -&gt; 247% (L10)
-Petrify: 20% (+1-2%/Lv) -&gt; 35% | TP Cost: 9 (+3-5/Lv) -&gt; 42 | Speed: 0.85x -&gt; 0.95x</t>
+          <t>ATK: 135% (+11-14%/Lv) -&gt; 247% | Petrify: 20% (+1-2%/Lv) -&gt; 35% | Accuracy: +10%
+TP Cost: 9 -&gt; 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 37 -&gt; 42</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1754,10 +1766,14 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Petrify, TP Cost</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr"/>
+          <t>ATK, Petrify</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr">
         <is>
           <t>Axe skill. Strike one enemy with earth damage. May petrify.</t>
@@ -2021,7 +2037,7 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>ATK: 130% -&gt; 140 -&gt; 150 -&gt; 160 -&gt; 170 -&gt; 180 -&gt; 190 -&gt; 200 -&gt; 211 -&gt; 222% (L10)
-Accuracy: +6% (+1-2%/Lv) -&gt; +20% | TP Cost: 12 (+3/Lv) -&gt; 39 | Speed: 0.8x -&gt; 0.9x</t>
+Accuracy: +6% -&gt; +20% | Damage vs. unholy: +65% | TP Cost: 12 (+3/Lv) -&gt; 39</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -2037,7 +2053,11 @@
           <t>Accuracy</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>Sword and lance skill. Strike one enemy. Effective vs. Unholy foes.</t>
@@ -2083,7 +2103,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Shield skill. Reduce physical damage taken by the party once.</t>
+          <t>Shield skill. Reduce physical damage taken by the party once (12-30%).</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2151,7 +2171,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Shield skill. Reduce magic damage taken by the party once.</t>
+          <t>Shield skill. Reduce magic damage taken by the party once (12-30%).</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2297,7 +2317,7 @@
       <c r="H27" t="inlineStr">
         <is>
           <t>ATK: 135% -&gt; 149 -&gt; 163 -&gt; 176 -&gt; 189 -&gt; 201 -&gt; 213 -&gt; 223 -&gt; 234 -&gt; 245% (L10)
-Silence: 20% (+3-4%/Lv) -&gt; 50% | TP Cost: 7 (+3/Lv) -&gt; 34 | Speed: 0.85x -&gt; 0.95x</t>
+Silence: 20% (+3-4%/Lv) -&gt; 50% | Accuracy: +15% | TP Cost: 7 (+3/Lv) -&gt; 34</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -2313,7 +2333,11 @@
           <t>Silence</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>Lance skill. Strike one enemy with wind damage. May silence.</t>
@@ -2365,7 +2389,7 @@
       <c r="H28" t="inlineStr">
         <is>
           <t>ATK: 116% -&gt; 118 -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 146 -&gt; 152% (L10)
-TP Cost: 36 -&gt; 39 -&gt; 42 -&gt; 45 -&gt; 48 -&gt; 51 -&gt; 55 -&gt; 59 -&gt; 65 -&gt; 71</t>
+Heavy Lance bonus: +20% | TP Cost: 36 (+3-6/Lv) -&gt; 71 | Speed: 0.7x -&gt; 0.8x</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -2376,12 +2400,12 @@
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
           <t>Lance skill. Rapidly strike random enemies 3 to 5 times.</t>
@@ -2495,7 +2519,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deal increased physical damage next turn.</t>
+          <t>Deal increased physical damage next turn (1.05-1.3x).</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2558,7 +2582,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Steal pocket money from an enemy.</t>
+          <t>Steal pocket money from an enemy (Steal success 40-64%).</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2621,7 +2645,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Steal an item from an enemy.</t>
+          <t>Steal an item from an enemy (Steal success 30-50%).</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2813,7 +2837,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Increase own physical evasion rate.</t>
+          <t>Increase own physical evasion rate (10%+).</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2945,7 +2969,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Increase own accuracy.</t>
+          <t>Increase own accuracy (15-30%).</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3017,7 +3041,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Increase own speed.</t>
+          <t>Increase own speed (10%+).</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3115,7 +3139,11 @@
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 104 characters</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3494,26 +3522,18 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Damage UP
-TP Cost: 42 -&gt; 50 -&gt; 57 -&gt; 63 -&gt; 68 (L1-5 Max) | Speed: 0.4x</t>
+          <t>Damage: 3.3x -&gt; 3.45x -&gt; 3.6x -&gt; 3.8x -&gt; 4x (L1-5 Max) | ATK: 88%
+TP Cost: 42 -&gt; 50 -&gt; 57 -&gt; 63 -&gt; 68 | Speed: 0.4x</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Damage UP</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>effect_2</t>
-        </is>
-      </c>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr">
@@ -4050,8 +4070,8 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>ATK: 94% -&gt; 97 -&gt; 100 -&gt; 103 -&gt; 106 -&gt; 110 -&gt; 114 -&gt; 119 -&gt; 124 -&gt; 130% (L10)
-Speed decrease chance: 30% (+5%/Lv) | Turns: 4 | TP Cost: 24 (+2-3/Lv) -&gt; 50</t>
+          <t>ATK: 94% (+3-6%/Lv) -&gt; 130% | Speed decrease chance: 30% -&gt; 75% | Speed decrease: 10%
+Turns: 4 | TP Cost: 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 39 -&gt; 42 -&gt; 45 -&gt; 48 -&gt; 50</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -4064,7 +4084,7 @@
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
-          <t>TP Cost</t>
+          <t>ATK, Speed decrease chance</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4179,7 +4199,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Identify unknown items.</t>
+          <t>Identify unknown items (Identification success rate 32-80%).</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -4268,7 +4288,11 @@
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 100 characters</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4307,32 +4331,28 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Damage UP | Accuracy: +10% (+2-4%/Lv) -&gt; +30%
-TP Cost: 28 -&gt; 32 -&gt; 36 -&gt; 40 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 56 -&gt; 60 -&gt; 64 | Speed: 0.75x</t>
+          <t>Damage: 2x -&gt; 2.2 -&gt; 2.4 -&gt; 2.6 -&gt; 2.8 -&gt; 3 -&gt; 3.25 -&gt; 3.5 -&gt; 3.75 -&gt; 4x (L10)
+Accuracy: +10% (+2-4%/Lv) -&gt; +30% | ATK: 82% | TP Cost: 28 (+4/Lv) -&gt; 64</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Damage UP</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>effect_3</t>
-        </is>
-      </c>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>Accuracy</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
       <c r="O57" t="inlineStr">
         <is>
           <t>Mace skill. Heavy bash strike with boosted accuracy.</t>
@@ -4387,7 +4407,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>ATK: 135% -&gt; 147 -&gt; 159 -&gt; 171 -&gt; 183 -&gt; 193 -&gt; 203 -&gt; 213 -&gt; 220 -&gt; 225% (L10)
+          <t>ATK: 135% -&gt; 147 -&gt; 159 -&gt; 171 -&gt; 183 -&gt; 193 -&gt; 203 -&gt; 213 -&gt; 220 -&gt; 225% | DEF: -10%
 Turns: 4 | TP Cost: 25 -&gt; 29 -&gt; 33 -&gt; 37 -&gt; 41 -&gt; 45 -&gt; 48 -&gt; 51 -&gt; 54 -&gt; 57</t>
         </is>
       </c>
@@ -4518,7 +4538,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Reduce magic damage taken for the party.</t>
+          <t>Reduce magic damage taken for the party (18-36%).</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4581,7 +4601,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Transform to increase own overall stats.</t>
+          <t>Transform to increase own overall stats (20-32%).</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4871,7 +4891,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Heal an ally's HP.</t>
+          <t>Heal an ally's HP (HP recovery 12-25%).</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -4933,7 +4953,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Heal an ally's TP.</t>
+          <t>Heal an ally's TP (TP recovery 10%+).</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4996,7 +5016,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Distribute all of one's TP to the target.</t>
+          <t>Distribute all of one's TP to the target (TP transfer bonus 100-140%).</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -5058,7 +5078,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Clean one's surroundings in order to increase mobility.</t>
+          <t>Clean one's surroundings in order to increase mobility (Speed increase 12%+).</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -5121,7 +5141,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Recover some TP.</t>
+          <t>Recover some TP (16%+).</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -5184,7 +5204,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Dance skill. Lower all enemies' ATK while dance lasts.</t>
+          <t>Dance skill. Lower all enemies' ATK while dance lasts (4-16%).</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -5247,7 +5267,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Dance skill. Lower all enemies' DEF while dance lasts.</t>
+          <t>Dance skill. Lower all enemies' DEF while dance lasts (5-23%).</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -5310,7 +5330,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Dance skill. Lower all enemies' accuracy while dance lasts.</t>
+          <t>Dance skill. Lower all enemies' accuracy while dance lasts (4%+).</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -5364,7 +5384,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Dance skill. Lower all enemies' evasion while dance lasts.</t>
+          <t>Dance skill. Lower all enemies' evasion while dance lasts (5-23%).</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -5444,7 +5464,11 @@
       </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
-      <c r="Q75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 124 characters</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5477,7 +5501,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Dance skill. Lower all enemies' speed while dance lasts.</t>
+          <t>Dance skill. Lower all enemies' speed while dance lasts (5%+).</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -5531,7 +5555,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Dance skill. Lower all enemies' elemental resistances while dance lasts.</t>
+          <t>Dance skill. Lower all enemies' elemental resistances while dance lasts (7-25%).</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -5592,7 +5616,7 @@
       <c r="H78" t="inlineStr">
         <is>
           <t>ATK: 120% -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 145 -&gt; 150 -&gt; 155 -&gt; 160% (L10)
-TP Cost: 22 -&gt; 25 -&gt; 28 -&gt; 31 -&gt; 34 -&gt; 37 -&gt; 40 -&gt; 43 -&gt; 46 -&gt; 50</t>
+Power decrease: 10% | TP Cost: 22 (+3-4/Lv) -&gt; 50 | Speed: 0.75x -&gt; 0.85x</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -5603,12 +5627,12 @@
       </c>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr">
         <is>
           <t>Whip skill. Deal bash damage to an enemy row from mid-range.</t>
@@ -5778,7 +5802,7 @@
       <c r="H81" t="inlineStr">
         <is>
           <t>ATK: 104% -&gt; 108 -&gt; 112 -&gt; 116 -&gt; 120 -&gt; 124 -&gt; 127 -&gt; 130 -&gt; 133 -&gt; 136% (L10)
-TP Cost: 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 40 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 56 -&gt; 60</t>
+Accuracy: +20% | TP Cost: 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 40 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 56 -&gt; 60</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -5840,7 +5864,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Take a break to heal own HP and raise Pep.</t>
+          <t>Take a break to heal own HP and raise Pep (HP recovery 20-40%).</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -6076,7 +6100,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Increase own ATK at the price of lowering own DEF.</t>
+          <t>Increase own ATK at the price of lowering own DEF (ATK 15-35%, DEF 11-25%).</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -6210,7 +6234,11 @@
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 94 characters</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6547,7 +6575,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Convert current DEF to bonus ATK (DEF becomes 0).</t>
+          <t>Convert current DEF to bonus ATK (DEF becomes 0) (60-150%).</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -6723,7 +6751,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Summon Spartan for short-range bash damage.</t>
+          <t>Summon Spartan for short-range bash damage (Duration 3-6).</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -6799,7 +6827,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Summon Oracles for mid-range INT-based damage and possible paralysis.</t>
+          <t>Summon Oracles for mid-range INT-based damage and possible paralysis (Duration 3-5).</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -6862,7 +6890,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Summon Catalina to heal allies' HP.</t>
+          <t>Summon Catalina to heal allies' HP (Duration 3-5).</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -6934,7 +6962,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Summon Mercidarian for random long-range stab damage to all foes.</t>
+          <t>Summon Mercidarian for random long-range stab damage to all foes (Duration 2-4).</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -10849,7 +10877,7 @@
       <c r="H165" t="inlineStr">
         <is>
           <t>Pwr: 60 -&gt; 95 -&gt; 130 -&gt; 165 -&gt; 200 -&gt; 230 -&gt; 260 -&gt; 290 -&gt; 320 -&gt; 350 (L10)
-Accuracy: 80% (+1-2%/Lv) -&gt; 90% | TP Cost: 9 (+1/Lv) -&gt; 18 | Speed: 2x</t>
+Accuracy: 80% (+1-2%/Lv) -&gt; 90% | HP Absorb: 100% | TP Cost: 9 (+1/Lv) -&gt; 18</t>
         </is>
       </c>
       <c r="I165" t="inlineStr"/>
@@ -10867,7 +10895,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>Chant</t>
+          <t>Speed, Chant</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -10921,7 +10949,7 @@
       <c r="H166" t="inlineStr">
         <is>
           <t>Pwr: 22 -&gt; 30 -&gt; 38 -&gt; 46 -&gt; 54 -&gt; 60 -&gt; 66 -&gt; 72 -&gt; 78 -&gt; 82 | Accuracy: 80% -&gt; 90%
-TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15 | Speed: 1.75x</t>
+TP Absorb: 100% | TP Cost: 6 (+1/Lv) -&gt; 15 | Speed: 1.75x | Chant: 1.25x -&gt; 1.07x</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -10937,11 +10965,7 @@
           <t>Accuracy</t>
         </is>
       </c>
-      <c r="N166" t="inlineStr">
-        <is>
-          <t>Chant</t>
-        </is>
-      </c>
+      <c r="N166" t="inlineStr"/>
       <c r="O166" t="inlineStr">
         <is>
           <t>Neutral magic strike to one enemy. Absorb damage dealt as TP.</t>
@@ -10987,7 +11011,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Raise max HP.</t>
+          <t>Raise max HP (20-50%).</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -11060,8 +11084,8 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Pwr: 75 -&gt; 120 -&gt; 165 -&gt; 210 -&gt; 255 -&gt; 295 -&gt; 335 -&gt; 375 -&gt; 415 -&gt; 450 (L10)
-Accuracy: 65% (+2-3%/Lv) -&gt; 87% | TP Cost: 18 (+3-4/Lv) -&gt; 50 | Speed: 1.5x</t>
+          <t>Pwr: 75 (+35-45/Lv) -&gt; 450 | Accuracy: 65% (+2-3%/Lv) -&gt; 87% | HP Absorb: 100%
+TP Cost: 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 | Speed: 1.5x</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -11074,7 +11098,7 @@
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr">
         <is>
-          <t>Accuracy, TP Cost</t>
+          <t>Pwr, Accuracy</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11767,12 +11791,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Negate buffs for all enemies.</t>
+          <t>Negate buffs for all enemies (Accuracy 55-95%, Buff cancel rate 100%).</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Accuracy: 55% -&gt; 65% -&gt; 75% -&gt; 85% -&gt; 95% (L1-5 Max)
+          <t>Accuracy: 55% -&gt; 65% -&gt; 75% -&gt; 85% -&gt; 95% (L1-5 Max) | Buff cancel rate: 100%
 TP Cost: 8 -&gt; 11 -&gt; 14 -&gt; 18 -&gt; 22 | Speed: 1.25x | Chant: 1.25x -&gt; 1.45x</t>
         </is>
       </c>
@@ -11827,8 +11851,8 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Pwr: 250 -&gt; 300 -&gt; 350 -&gt; 400 -&gt; 440 -&gt; 480 -&gt; 520 -&gt; 560 -&gt; 600 -&gt; 640 (L10)
-Accuracy: 60% (+1-2%/Lv) -&gt; 70% | TP Cost: 45 (+4-8/Lv) -&gt; 100 | Speed: 1.75x</t>
+          <t>Pwr: 250 (+40-50/Lv) -&gt; 640 | Accuracy: 60% -&gt; 70% | Damage vs. unholy: +100%
+TP Cost: 45 -&gt; 52 -&gt; 59 -&gt; 66 -&gt; 74 -&gt; 80 -&gt; 86 -&gt; 90 -&gt; 95 -&gt; 100 | Speed: 1.75x</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -11841,7 +11865,7 @@
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="inlineStr">
         <is>
-          <t>Accuracy, TP Cost</t>
+          <t>Pwr, Accuracy</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -12205,7 +12229,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Raise one row of allies' resistance to stab damage.</t>
+          <t>Raise one row of allies' resistance to stab damage (20-36%).</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -12273,7 +12297,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Raise one row of allies' resistance to slash damage.</t>
+          <t>Raise one row of allies' resistance to slash damage (18-36%).</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -12341,7 +12365,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Raise one row of allies' resistance to bash damage.</t>
+          <t>Raise one row of allies' resistance to bash damage (18-36%).</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -12409,7 +12433,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Heal an ally's HP.</t>
+          <t>Heal an ally's HP (HP recovery 8-26, Heal Cap 100-800).</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -12481,7 +12505,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Heal the party's HP.</t>
+          <t>Heal the party's HP (HP recovery 5-14, Heal Cap 80-600).</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -12743,7 +12767,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Revive a dead ally.</t>
+          <t>Revive a dead ally (HP on revival 40-88%).</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -12807,7 +12831,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Raise an ally's ATK.</t>
+          <t>Raise an ally's ATK (10-22%).</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -12875,7 +12899,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Raise an ally's DEF.</t>
+          <t>Raise an ally's DEF (10-25%).</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -12943,7 +12967,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Raise the party's magic defense.</t>
+          <t>Raise the party's magic defense (10%+).</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -13011,7 +13035,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Raise the party's resistance to fire, water, lightning, wind, and earth.</t>
+          <t>Raise the party's resistance to fire, water, lightning, wind, and earth (5-25%).</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -13079,7 +13103,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Raise an ally's speed.</t>
+          <t>Raise an ally's speed (8%+).</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -13147,7 +13171,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Raise an ally's max HP.</t>
+          <t>Raise an ally's max HP (20-47%).</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -13343,7 +13367,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>Reduce incoming physical damage by a certain amount.</t>
+          <t>Reduce incoming physical damage by a certain amount (30-45%).</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -13407,7 +13431,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>While active, immediately revive upon death.</t>
+          <t>While active, immediately revive upon death (Amount of HP on revival 10-50%).</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -13701,7 +13725,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Raise the party's critical rate while song lasts.</t>
+          <t>Raise the party's critical rate while song lasts (10-28%).</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -13755,7 +13779,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Raise the party's magic attack power while song lasts.</t>
+          <t>Raise the party's magic attack power while song lasts (10%+).</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -13809,7 +13833,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Raise the party's magic defense power while song lasts.</t>
+          <t>Raise the party's magic defense power while song lasts (10%+).</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -13863,7 +13887,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Decrease the party's chant time while song lasts.</t>
+          <t>Decrease the party's chant time while song lasts (10%+).</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -13917,7 +13941,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Gradually heal the party's HP while song lasts.</t>
+          <t>Gradually heal the party's HP while song lasts (HP recovery 20-250).</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -13980,7 +14004,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Gradually heal the party's TP while song lasts.</t>
+          <t>Gradually heal the party's TP while song lasts (TP recovery 4-30).</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -14043,7 +14067,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Raise the party's speed while song lasts.</t>
+          <t>Raise the party's speed while song lasts (6%+).</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -14106,7 +14130,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Raise the party's acquired EXP while song lasts.</t>
+          <t>Raise the party's acquired EXP while song lasts (16%+).</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -14169,7 +14193,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Raise the party's magic accuracy while song lasts.</t>
+          <t>Raise the party's magic accuracy while song lasts (6%+).</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -14224,7 +14248,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Dodge enemy attacks by creating a shadow clone.</t>
+          <t>Dodge enemy attacks by creating a shadow clone (Number of dodges 1-5).</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -14304,7 +14328,11 @@
       <c r="N219" t="inlineStr"/>
       <c r="O219" t="inlineStr"/>
       <c r="P219" t="inlineStr"/>
-      <c r="Q219" t="inlineStr"/>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 95 characters</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -14338,7 +14366,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>Lower all enemies' accuracy.</t>
+          <t>Lower all enemies' accuracy (10%+).</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -14422,7 +14450,11 @@
       </c>
       <c r="O221" t="inlineStr"/>
       <c r="P221" t="inlineStr"/>
-      <c r="Q221" t="inlineStr"/>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 137 characters</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -14485,7 +14517,11 @@
       </c>
       <c r="O222" t="inlineStr"/>
       <c r="P222" t="inlineStr"/>
-      <c r="Q222" t="inlineStr"/>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 157 characters</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -14548,7 +14584,11 @@
       </c>
       <c r="O223" t="inlineStr"/>
       <c r="P223" t="inlineStr"/>
-      <c r="Q223" t="inlineStr"/>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 155 characters</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -14611,7 +14651,11 @@
       </c>
       <c r="O224" t="inlineStr"/>
       <c r="P224" t="inlineStr"/>
-      <c r="Q224" t="inlineStr"/>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 145 characters</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -14674,7 +14718,11 @@
       </c>
       <c r="O225" t="inlineStr"/>
       <c r="P225" t="inlineStr"/>
-      <c r="Q225" t="inlineStr"/>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 138 characters</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -14830,7 +14878,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Raise the party's ATK.</t>
+          <t>Raise the party's ATK (8%+).</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -14898,7 +14946,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Raise the party's DEF.</t>
+          <t>Raise the party's DEF (8%+).</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -14966,7 +15014,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Create a field that reduces damage for both sides for a time.</t>
+          <t>Create a field that reduces damage for both sides for a time (25%+).</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -15081,31 +15129,35 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>HP recovery UP | Recoverable status ailments UP
-HP on revival: 10% -&gt; 15 -&gt; 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 -&gt; 50% | Chant: 2.5x</t>
+          <t>HP recovery: 22 -&gt; 26 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 (L8)
+Recoverable status ailments: 1 (+1/Lv) | HP on revival: 10% (+5-10%/Lv) -&gt; 50%</t>
         </is>
       </c>
       <c r="I232" t="inlineStr"/>
       <c r="J232" t="inlineStr">
         <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="K232" t="inlineStr">
-        <is>
-          <t>HP recovery UP; Recoverable status ailments UP</t>
-        </is>
-      </c>
-      <c r="L232" t="inlineStr">
-        <is>
-          <t>effect_1, effect_2</t>
-        </is>
-      </c>
-      <c r="M232" t="inlineStr"/>
-      <c r="N232" t="inlineStr"/>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr"/>
+      <c r="L232" t="inlineStr"/>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>HP on revival</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>Chant</t>
+        </is>
+      </c>
       <c r="O232" t="inlineStr"/>
       <c r="P232" t="inlineStr"/>
-      <c r="Q232" t="inlineStr"/>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 164 characters</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -15168,7 +15220,11 @@
       </c>
       <c r="O233" t="inlineStr"/>
       <c r="P233" t="inlineStr"/>
-      <c r="Q233" t="inlineStr"/>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 126 characters</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -15729,7 +15785,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>ATK bonus with sword equipped.</t>
+          <t>ATK bonus with sword equipped (3-15%).</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -15791,7 +15847,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>ATK bonus with axe equipped.</t>
+          <t>ATK bonus with axe equipped (3-15%).</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -15853,7 +15909,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>ATK bonus with dagger equipped.</t>
+          <t>ATK bonus with dagger equipped (3-17%).</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -15915,7 +15971,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>ATK bonus with mace equipped.</t>
+          <t>ATK bonus with mace equipped (3-15%).</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -15977,7 +16033,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>ATK bonus with lance equipped.</t>
+          <t>ATK bonus with lance equipped (3-15%).</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -16039,7 +16095,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>ATK bonus with bow equipped.</t>
+          <t>ATK bonus with bow equipped (3-15%).</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -16101,7 +16157,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>ATK bonus with katana equipped.</t>
+          <t>ATK bonus with katana equipped (3-15%).</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -16163,7 +16219,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>ATK bonus with projectile weapon equipped.</t>
+          <t>ATK bonus with projectile weapon equipped (5-20%).</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -16225,7 +16281,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>ATK bonus with whip equipped.</t>
+          <t>ATK bonus with whip equipped (3-17%).</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -16287,7 +16343,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>ATK bonus with fan equipped.</t>
+          <t>ATK bonus with fan equipped (5-20%).</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -16349,7 +16405,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>ATK bonus for all weapons.</t>
+          <t>ATK bonus for all weapons (2%+).</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -16411,7 +16467,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>Magic attack power bonus.</t>
+          <t>Magic attack power bonus (6%+).</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -16473,30 +16529,23 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>Healing magic bonus. Raises healing cap.</t>
+          <t>Healing magic bonus. Raises healing cap (HP recovery bonus 8-26%, Heal Cap 10-100%).</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>LvUp: HP recovery bonus UP Recovery cap UP</t>
+          <t>HP recovery bonus: 8% -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26% (L10)
+Heal Cap: +10% -&gt; +20 -&gt; +30 -&gt; +40 -&gt; +50 -&gt; +60 -&gt; +70 -&gt; +80 -&gt; +90 -&gt; +100%</t>
         </is>
       </c>
       <c r="I255" t="inlineStr"/>
       <c r="J255" t="inlineStr">
         <is>
-          <t>Unchanged</t>
-        </is>
-      </c>
-      <c r="K255" t="inlineStr">
-        <is>
-          <t>HP recovery bonus UP; Recovery cap UP</t>
-        </is>
-      </c>
-      <c r="L255" t="inlineStr">
-        <is>
-          <t>effect_1, effect_2</t>
-        </is>
-      </c>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="inlineStr"/>
       <c r="M255" t="inlineStr"/>
       <c r="N255" t="inlineStr"/>
       <c r="O255" t="inlineStr">
@@ -16543,7 +16592,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>Recover HP every turn during battle.</t>
+          <t>Recover HP every turn during battle (2%+).</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -16605,7 +16654,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>Slightly recover HP every turn during battle.</t>
+          <t>Slightly recover HP every turn during battle (1%+).</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -16667,7 +16716,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>Recover TP every turn during battle.</t>
+          <t>Recover TP every turn during battle (3-16).</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -16729,7 +16778,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Slightly recover TP every turn during battle.</t>
+          <t>Slightly recover TP every turn during battle (1-9).</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -16791,7 +16840,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>Raise resistance to all elements.</t>
+          <t>Raise resistance to all elements (6%+).</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -16853,7 +16902,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>Occasionally counterattack after receiving physical damage.</t>
+          <t>Occasionally counterattack after receiving physical damage (6-18%).</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -16915,7 +16964,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Occasionally parry and counterattack when targeted by an enemy.</t>
+          <t>Occasionally parry and counterattack when targeted by an enemy (Activation rate 4%+).</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -16977,7 +17026,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Occasionally attack twice when attacking normally.</t>
+          <t>Occasionally attack twice when attacking normally (Double attack rate 9-21%).</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -17039,7 +17088,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Occasionally attack thrice when attacking normally.</t>
+          <t>Occasionally attack thrice when attacking normally (Triple attack rate 5-17%).</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -17101,7 +17150,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Increase evasion rate against stab attacks.</t>
+          <t>Increase evasion rate against stab attacks (20-36%).</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -17154,7 +17203,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Occasionally parry when receiving long-range attacks.</t>
+          <t>Occasionally parry when receiving long-range attacks (Activation rate 10-30%).</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -17207,7 +17256,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Occasionally survive at 1 HP after being dealt fatal damage.</t>
+          <t>Occasionally survive at 1 HP after being dealt fatal damage (10-30%).</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -17269,7 +17318,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Occasionally Defend automatically when receiving physical attacks.</t>
+          <t>Occasionally Defend automatically when receiving physical attacks (4%+).</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -17331,7 +17380,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Can equip two one-handed weapons at the same time.</t>
+          <t>Can equip two one-handed weapons at the same time (Sub-weapon ATK 30-72%).</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -17393,7 +17442,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>Convert some received damage to TP.</t>
+          <t>Convert some received damage to TP (4-20%).</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -17446,7 +17495,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Occasionally instakill when inflicting a critical hit.</t>
+          <t>Occasionally instakill when inflicting a critical hit (Activation rate 8-20%).</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -17499,7 +17548,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>With bow equipped, occasionally halt an enemy's action.</t>
+          <t>With bow equipped, occasionally halt an enemy's action (Activation rate 2%+).</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -17572,7 +17621,11 @@
       <c r="N273" t="inlineStr"/>
       <c r="O273" t="inlineStr"/>
       <c r="P273" t="inlineStr"/>
-      <c r="Q273" t="inlineStr"/>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 90 characters</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -17605,7 +17658,7 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>Gain increased speed based on missing HP.</t>
+          <t>Gain increased speed based on missing HP (15%+).</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -17658,7 +17711,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Debuff an enemy when they inflict short-range damage.</t>
+          <t>Debuff an enemy when they inflict short-range damage (1-6).</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -17711,7 +17764,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>Increase ATK while inflicted with status ailments.</t>
+          <t>Increase ATK while inflicted with status ailments (15-27%).</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -17854,7 +17907,7 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Decrease physical damage to the back row when using a shield in the front row.</t>
+          <t>Decrease physical damage to the back row when using a shield in the front row (6%+).</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
@@ -17907,7 +17960,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Occasionally nullify physical damage.</t>
+          <t>Occasionally nullify physical damage (Activation rate 8%+).</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
@@ -17984,11 +18037,7 @@
         </is>
       </c>
       <c r="K281" t="inlineStr"/>
-      <c r="L281" t="inlineStr">
-        <is>
-          <t>effect_1</t>
-        </is>
-      </c>
+      <c r="L281" t="inlineStr"/>
       <c r="M281" t="inlineStr"/>
       <c r="N281" t="inlineStr"/>
       <c r="O281" t="inlineStr">
@@ -18035,7 +18084,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Briefly increase ATK and DEX when HP drops below 50%.</t>
+          <t>Briefly increase ATK and DEX when HP drops below 50% (10%+).</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
@@ -18097,7 +18146,7 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Make it harder for chants, songs, and dances to be interrupted.</t>
+          <t>Make it harder for chants, songs, and dances to be interrupted (10-50%).</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
@@ -18158,7 +18207,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Reduce chant time.</t>
+          <t>Reduce chant time (8-20%).</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
@@ -18220,7 +18269,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Reduce TP Cost in battle.</t>
+          <t>Reduce TP Cost in battle (10-30%).</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -18282,7 +18331,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Heighten magic accuracy.</t>
+          <t>Heighten magic accuracy (3%+).</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
@@ -18344,7 +18393,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Limit enemies' preemptive attacks.</t>
+          <t>Limit enemies' preemptive attacks (Enemy preemptive attack rate 20-50%).</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
@@ -18406,7 +18455,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Increase party's preemptive attack rate.</t>
+          <t>Increase party's preemptive attack rate (8-20%).</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
@@ -18468,7 +18517,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>May escape from battle more easily.</t>
+          <t>May escape from battle more easily (20-40%).</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
@@ -18530,7 +18579,7 @@
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>Increase the enemies' item drop rate.</t>
+          <t>Increase the enemies' item drop rate (4%+).</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
@@ -18592,7 +18641,7 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>Increase the amount of money the enemies drop.</t>
+          <t>Increase the amount of money the enemies drop (Gold drop rate 25-125%).</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
@@ -18654,7 +18703,7 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>Sometimes pick up items while moving around the dungeons.</t>
+          <t>Sometimes pick up items while moving around the dungeons (Found item quality 1-5).</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
@@ -18746,7 +18795,11 @@
 Restores whole party after combat conclusion</t>
         </is>
       </c>
-      <c r="Q293" t="inlineStr"/>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>values left out: the sentence would be 95 characters</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -18779,7 +18832,7 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>Occasionally keep disposable items after using them in battle.</t>
+          <t>Occasionally keep disposable items after using them in battle (25%+).</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
@@ -18841,7 +18894,7 @@
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>Increase the effects of HP and TP recovery items during battle.</t>
+          <t>Increase the effects of HP and TP recovery items during battle (10-100%).</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
@@ -18903,7 +18956,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>Become capable of performing two songs at once.</t>
+          <t>Become capable of performing two songs at once (Speed 6-18%).</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -18965,7 +19018,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Become capable of performing two dances at once.</t>
+          <t>Become capable of performing two dances at once (Speed 6-18%).</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
@@ -19027,7 +19080,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>Become capable of controlling two dolls at once.</t>
+          <t>Become capable of controlling two dolls at once (Speed 6-18%).</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
@@ -19089,7 +19142,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>Increase doll power with the strength of the equipped Sealbook.</t>
+          <t>Increase doll power with the strength of the equipped Sealbook (15-27%).</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
@@ -19151,7 +19204,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>Increased effects for all maid skills.</t>
+          <t>Increased effects for all maid skills (1%+).</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
@@ -19213,7 +19266,7 @@
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>Increased effects for all songs.</t>
+          <t>Increased effects for all songs (Singing skill bonus 3%+).</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
@@ -19275,7 +19328,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>Increased effects for all dances.</t>
+          <t>Increased effects for all dances (Dancing skill bonus 3%+).</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
@@ -19337,7 +19390,7 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>Increased effects for all doll skills.</t>
+          <t>Increased effects for all doll skills (3%+).</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
@@ -19399,7 +19452,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>Occasionally attack twice when attacking normally.</t>
+          <t>Occasionally attack twice when attacking normally (Double attack rate 20-32%).</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
@@ -19461,7 +19514,7 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>Reduce chant time for songs.</t>
+          <t>Reduce chant time for songs (10%+).</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
@@ -19523,7 +19576,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>Reduce purchase and identification prices at shops.</t>
+          <t>Reduce purchase and identification prices at shops (Negotiation rate 10-25%).</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
@@ -19585,7 +19638,7 @@
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>Mesmerize enemies, causing them to occasionally do nothing.</t>
+          <t>Mesmerize enemies, causing them to occasionally do nothing (Occurrence rate 3%+).</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
@@ -20919,19 +20972,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C2" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E2" t="n">
         <v>18</v>
       </c>
       <c r="F2" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3">
@@ -20941,10 +20994,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -20953,7 +21006,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -20991,13 +21044,13 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
qol: refine doll turns to stepped level ranges and document x86 reverse
refine doll turns to stepped level ranges and document x86 reverse
engineering of 144 enchants

- Dolls (Spartan, Oracles, Catalina, Mercidarian, Star Dust Arrow):
display stepped turn ranges e.g. 'Turns: 3 (Lv1-3) -> 4 (Lv4-6) -> 5
(Lv7-9) -> 6 (L10)' for instant readability while preserving combat
progression on Line 2. - text_checks.py: support monotonic stepped
series matching in series_fits() and fallback to summon turns (effect
147) for Turns label. - test_effect_decoding.py: update assertions to
verify stepped turns notation. - docs/ENCHANT_ANALYSIS_ROADMAP_B.md:
complete reverse engineering report on 144 equipment enchantments from
x86 disassembly.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_skill_text.xlsx
+++ b/mod_project/data_tables/qol_skill_text.xlsx
@@ -3113,7 +3113,7 @@
       <c r="H51" t="inlineStr">
         <is>
           <t>ATK: 100% -&gt; 102 -&gt; 104 -&gt; 106 -&gt; 108 -&gt; 110 -&gt; 112 -&gt; 114 -&gt; 117 -&gt; 120% (L10)
-1-3 hits   |   Duration: 2 -&gt; 3   |   TP Cost: 35 (+3/Lv) -&gt; 62   |   Speed: 0.82x</t>
+1-3 hits   |   Turns: 2 (Lv1-9) -&gt; 3 (L10 Max)   |   TP Cost: 35 (+3/Lv) -&gt; 62</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5352,7 +5352,7 @@
       <c r="H97" t="inlineStr">
         <is>
           <t>ATK: 144% -&gt; 147 -&gt; 150 -&gt; 154 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170 -&gt; 175 -&gt; 180% (L10)
-Duration: 3 -&gt; 6   |   TP Cost: 20 (+2-3/Lv) -&gt; 42   |   Speed: 0.85x -&gt; 0.98x</t>
+Turns: 3 (Lv1-3) -&gt; 4 (Lv4-6) -&gt; 5 (Lv7-9) -&gt; 6 (L10)   |   TP Cost: 20 -&gt; 42</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5409,7 +5409,7 @@
       <c r="H98" t="inlineStr">
         <is>
           <t>ATK: 126% (+2-5%/Lv) -&gt; 157%   |   Paralysis: 30% (+3-5%/Lv) -&gt; 64% (L10)
-Duration: 3 -&gt; 5   |   TP Cost: 24 (+2-3/Lv) -&gt; 48   |   Speed: 0.9x</t>
+Turns: 3 (Lv1-4) -&gt; 4 (Lv5-8) -&gt; 5 (Lv9-10) | TP Cost: 24 -&gt; 48 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5460,8 +5460,8 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Heal Power: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12 (L1-5 Max)   |   Duration: 3 -&gt; 5
-TP Cost: 30 -&gt; 33 -&gt; 37 -&gt; 42 -&gt; 48   |   Speed: 0.9x</t>
+          <t>Heal Power: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12 (L1-5 Max)
+Turns: 3 (Lv1-2) -&gt; 4 (Lv3-4) -&gt; 5 (L5 Max) | TP Cost: 30 -&gt; 48 | Speed: 0.9x</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5513,7 +5513,7 @@
       <c r="H100" t="inlineStr">
         <is>
           <t>ATK: 100% -&gt; 104 -&gt; 108 -&gt; 112 -&gt; 118 -&gt; 123 -&gt; 128 -&gt; 133 -&gt; 138 -&gt; 143% (L10)
-Duration: 2 -&gt; 4   |   TP Cost: 42 (+2-6/Lv) -&gt; 70   |   Speed: 0.75x</t>
+Turns: 2 (Lv1-4) -&gt; 3 (Lv5-7) -&gt; 4 (Lv8-10) | TP Cost: 42 -&gt; 70 | Speed: 0.75x</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5612,7 +5612,7 @@
       <c r="H102" t="inlineStr">
         <is>
           <t>Pwr: 180 -&gt; 240 -&gt; 310 -&gt; 390 -&gt; 480 -&gt; 585 -&gt; 700 (L7 Max)
-Duration: 4   |   TP Cost: 38 (+4-6/Lv) -&gt; 68   |   Speed: 0.82x -&gt; 0.92x</t>
+Turns: 4   |   TP Cost: 38 (+4-6/Lv) -&gt; 68   |   Speed: 0.82x -&gt; 0.92x</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">

</xml_diff>

<commit_message>
qol: improve readability for stepped-turn and scroll skills
- Format stepped turn progressions into clean level ranges (Fleet Foot,
Megaton Press, Chain Spike) - Reorganize ninja scrolls (Wind, Fire,
Earth) to group 3-turn debuff duration with ailment effect - Refine
Carrot and Stick Line 3 parameters to fit comfortably under 85
characters - Retain exact vanilla TP progressions and cleansing priority
lists per user feedback - All 196 tests passing
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_skill_text.xlsx
+++ b/mod_project/data_tables/qol_skill_text.xlsx
@@ -1533,7 +1533,12 @@
       <c r="H20" t="inlineStr">
         <is>
           <t>ATK: 120% -&gt; 130 -&gt; 140 -&gt; 148 -&gt; 156 -&gt; 164 -&gt; 170 -&gt; 176 -&gt; 180 -&gt; 184% (L10)
-Targets: 2 -&gt; 2 -&gt; 2 -&gt; 3 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 5 -&gt; 5   |   TP Cost: 26 (+4-6/Lv) -&gt; 68</t>
+Targets: 2 (Lv1-3) -&gt; 3 (Lv4-6) -&gt; 4 (Lv7-8) -&gt; 5 (L9-10) | TP: 26 (+4-6/Lv) -&gt; 68</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2457,7 +2462,12 @@
       <c r="H38" t="inlineStr">
         <is>
           <t>Speed increase: 10% -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15 -&gt; 16 -&gt; 17 -&gt; 18 -&gt; 20% (L10)
-Turns: 3 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 5 -&gt; 5 -&gt; 5 -&gt; 6   |   TP Cost: 14 (+2/Lv) -&gt; 32</t>
+Turns: 3 (Lv1-3) -&gt; 4 (Lv4-6) -&gt; 5 (Lv7-9) -&gt; 6 (L10)  |  TP Cost: 14 (+2/Lv) -&gt; 32</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2711,8 +2721,13 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Number of attacks: 3 -&gt; 3 -&gt; 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 4 -&gt; 5 -&gt; 5   |   ATK: 104% -&gt; 148%
-Power decrease: 25% -&gt; 14%   |   TP Cost: 30 (+4-6/Lv) -&gt; 72   |   Speed: 0.75x -&gt; 0.85x</t>
+          <t>Number of attacks: 3 (Lv1-4) -&gt; 4 (Lv5-8) -&gt; 5 (L9-10)   |   ATK: 104% -&gt; 148%
+Power decrease: 25% -&gt; 14% | TP Cost: 30 (+4-6/Lv) -&gt; 72 | Speed: 0.75x -&gt; 0.85x</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -11452,7 +11467,12 @@
       <c r="H221" t="inlineStr">
         <is>
           <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
-ATK: -4% (-1%/Lv) | Damage cap: 250 -&gt; 500 | Turns: 3 | TP Cost: 20 (+5/Lv) -&gt; 40</t>
+ATK: -4% (-1%/Lv) (3 Turns) | Damage cap: 250 -&gt; 500 | TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -11623,7 +11643,12 @@
       <c r="H224" t="inlineStr">
         <is>
           <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
-Evasion: -7% (-2%/Lv) | Damage cap: 250 -&gt; 500 | Turns: 3 | TP Cost: 20 (+5/Lv) -&gt; 40</t>
+Evasion: -7% (-2%/Lv) (3 Turns) | Damage cap: 250 -&gt; 500 | TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
@@ -11680,7 +11705,12 @@
       <c r="H225" t="inlineStr">
         <is>
           <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
-DEF: -4% (-1%/Lv) | Damage cap: 250 -&gt; 500 | Turns: 3 | TP Cost: 20 (+5/Lv) -&gt; 40</t>
+DEF: -4% (-1%/Lv) (3 Turns) | Damage cap: 250 -&gt; 500 | TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -12101,7 +12131,12 @@
       <c r="H233" t="inlineStr">
         <is>
           <t>DEF: -5% -&gt; -6% -&gt; -7% -&gt; -8% -&gt; -10% (L1-5 Max)   |   Magic defense: -10% -&gt; -15%
-Accuracy: 80% -&gt; 90% | HP recovery: 35 -&gt; 25 | Turns: 3 | TP Cost: 18 (+2-4/Lv) -&gt; 32</t>
+Accuracy: 80% -&gt; 90% | HP recovery: 35 -&gt; 25 | Turns: 3 | TP: 18 (+2-4/Lv) -&gt; 32</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">

</xml_diff>